<commit_message>
weekly update, 2022-03-02, SARS-CoV-2
</commit_message>
<xml_diff>
--- a/pdb/nsp3/SARS-CoV-2/domains_and_infos_of_nsp3.xlsx
+++ b/pdb/nsp3/SARS-CoV-2/domains_and_infos_of_nsp3.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1771" uniqueCount="755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1776" uniqueCount="758">
   <si>
     <t>nsp3_Macro1_</t>
   </si>
@@ -2123,6 +2123,15 @@
   </si>
   <si>
     <t>2020-04-28</t>
+  </si>
+  <si>
+    <t>7tzj</t>
+  </si>
+  <si>
+    <t>SARS COV-2 PLPRO IN COMPLEX WITH INHIBITOR 3K</t>
+  </si>
+  <si>
+    <t>2022-02-15</t>
   </si>
   <si>
     <t>7sgv</t>
@@ -7531,7 +7540,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7553,19 +7562,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="B3">
         <v>2.72</v>
       </c>
       <c r="C3" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
     </row>
   </sheetData>
@@ -7585,7 +7594,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7607,19 +7616,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="B3">
         <v>2.68</v>
       </c>
       <c r="C3" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
     </row>
   </sheetData>
@@ -7639,7 +7648,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7661,13 +7670,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="B3">
         <v>3.21</v>
       </c>
       <c r="C3" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -7678,19 +7687,19 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="B4">
         <v>2.73</v>
       </c>
       <c r="C4" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
   </sheetData>
@@ -7700,7 +7709,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B349"/>
+  <dimension ref="A1:B350"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
@@ -7708,12 +7717,12 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -7721,7 +7730,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -7884,7 +7893,7 @@
     </row>
     <row r="35" spans="2:2">
       <c r="B35" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
     </row>
     <row r="36" spans="2:2">
@@ -7909,7 +7918,7 @@
     </row>
     <row r="40" spans="2:2">
       <c r="B40" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
     </row>
     <row r="41" spans="2:2">
@@ -7934,7 +7943,7 @@
     </row>
     <row r="45" spans="2:2">
       <c r="B45" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
     </row>
     <row r="46" spans="2:2">
@@ -7984,7 +7993,7 @@
     </row>
     <row r="55" spans="2:2">
       <c r="B55" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
     </row>
     <row r="56" spans="2:2">
@@ -8214,7 +8223,7 @@
     </row>
     <row r="101" spans="2:2">
       <c r="B101" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
     </row>
     <row r="102" spans="2:2">
@@ -8344,7 +8353,7 @@
     </row>
     <row r="127" spans="2:2">
       <c r="B127" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
     </row>
     <row r="128" spans="2:2">
@@ -8354,7 +8363,7 @@
     </row>
     <row r="129" spans="2:2">
       <c r="B129" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
     </row>
     <row r="130" spans="2:2">
@@ -8459,7 +8468,7 @@
     </row>
     <row r="150" spans="2:2">
       <c r="B150" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
     </row>
     <row r="151" spans="2:2">
@@ -8589,7 +8598,7 @@
     </row>
     <row r="176" spans="2:2">
       <c r="B176" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
     </row>
     <row r="177" spans="2:2">
@@ -8649,805 +8658,810 @@
     </row>
     <row r="188" spans="2:2">
       <c r="B188" t="s">
-        <v>649</v>
+        <v>699</v>
       </c>
     </row>
     <row r="189" spans="2:2">
       <c r="B189" t="s">
-        <v>337</v>
+        <v>649</v>
       </c>
     </row>
     <row r="190" spans="2:2">
       <c r="B190" t="s">
-        <v>652</v>
+        <v>337</v>
       </c>
     </row>
     <row r="191" spans="2:2">
       <c r="B191" t="s">
-        <v>338</v>
+        <v>652</v>
       </c>
     </row>
     <row r="192" spans="2:2">
       <c r="B192" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="193" spans="2:2">
       <c r="B193" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="194" spans="2:2">
       <c r="B194" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="195" spans="2:2">
       <c r="B195" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="196" spans="2:2">
       <c r="B196" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="197" spans="2:2">
       <c r="B197" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="198" spans="2:2">
       <c r="B198" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="199" spans="2:2">
       <c r="B199" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="200" spans="2:2">
       <c r="B200" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="201" spans="2:2">
       <c r="B201" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="202" spans="2:2">
       <c r="B202" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="203" spans="2:2">
       <c r="B203" t="s">
-        <v>654</v>
+        <v>361</v>
       </c>
     </row>
     <row r="204" spans="2:2">
       <c r="B204" t="s">
-        <v>363</v>
+        <v>654</v>
       </c>
     </row>
     <row r="205" spans="2:2">
       <c r="B205" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="206" spans="2:2">
       <c r="B206" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="207" spans="2:2">
       <c r="B207" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="208" spans="2:2">
       <c r="B208" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="209" spans="2:2">
       <c r="B209" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="210" spans="2:2">
       <c r="B210" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="211" spans="2:2">
       <c r="B211" t="s">
-        <v>657</v>
+        <v>374</v>
       </c>
     </row>
     <row r="212" spans="2:2">
       <c r="B212" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
     <row r="213" spans="2:2">
       <c r="B213" t="s">
-        <v>377</v>
+        <v>660</v>
       </c>
     </row>
     <row r="214" spans="2:2">
       <c r="B214" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="215" spans="2:2">
       <c r="B215" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="216" spans="2:2">
       <c r="B216" t="s">
-        <v>723</v>
+        <v>380</v>
       </c>
     </row>
     <row r="217" spans="2:2">
       <c r="B217" t="s">
-        <v>382</v>
+        <v>726</v>
       </c>
     </row>
     <row r="218" spans="2:2">
       <c r="B218" t="s">
-        <v>736</v>
+        <v>382</v>
       </c>
     </row>
     <row r="219" spans="2:2">
       <c r="B219" t="s">
-        <v>384</v>
+        <v>739</v>
       </c>
     </row>
     <row r="220" spans="2:2">
       <c r="B220" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="221" spans="2:2">
       <c r="B221" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="222" spans="2:2">
       <c r="B222" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="223" spans="2:2">
       <c r="B223" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="224" spans="2:2">
       <c r="B224" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="225" spans="2:2">
       <c r="B225" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="226" spans="2:2">
       <c r="B226" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="227" spans="2:2">
       <c r="B227" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="228" spans="2:2">
       <c r="B228" t="s">
-        <v>663</v>
+        <v>400</v>
       </c>
     </row>
     <row r="229" spans="2:2">
       <c r="B229" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
     </row>
     <row r="230" spans="2:2">
       <c r="B230" t="s">
-        <v>402</v>
+        <v>666</v>
       </c>
     </row>
     <row r="231" spans="2:2">
       <c r="B231" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="232" spans="2:2">
       <c r="B232" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="233" spans="2:2">
       <c r="B233" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="234" spans="2:2">
       <c r="B234" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="235" spans="2:2">
       <c r="B235" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="236" spans="2:2">
       <c r="B236" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="237" spans="2:2">
       <c r="B237" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="238" spans="2:2">
       <c r="B238" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="239" spans="2:2">
       <c r="B239" t="s">
-        <v>669</v>
+        <v>420</v>
       </c>
     </row>
     <row r="240" spans="2:2">
       <c r="B240" t="s">
-        <v>421</v>
+        <v>669</v>
       </c>
     </row>
     <row r="241" spans="2:2">
       <c r="B241" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="242" spans="2:2">
       <c r="B242" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="243" spans="2:2">
       <c r="B243" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="244" spans="2:2">
       <c r="B244" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="245" spans="2:2">
       <c r="B245" t="s">
-        <v>671</v>
+        <v>429</v>
       </c>
     </row>
     <row r="246" spans="2:2">
       <c r="B246" t="s">
-        <v>431</v>
+        <v>671</v>
       </c>
     </row>
     <row r="247" spans="2:2">
       <c r="B247" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="248" spans="2:2">
       <c r="B248" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="249" spans="2:2">
       <c r="B249" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="250" spans="2:2">
       <c r="B250" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="251" spans="2:2">
       <c r="B251" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="252" spans="2:2">
       <c r="B252" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="253" spans="2:2">
       <c r="B253" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="254" spans="2:2">
       <c r="B254" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="255" spans="2:2">
       <c r="B255" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="256" spans="2:2">
       <c r="B256" t="s">
-        <v>673</v>
+        <v>450</v>
       </c>
     </row>
     <row r="257" spans="2:2">
       <c r="B257" t="s">
-        <v>452</v>
+        <v>673</v>
       </c>
     </row>
     <row r="258" spans="2:2">
       <c r="B258" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="259" spans="2:2">
       <c r="B259" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="260" spans="2:2">
       <c r="B260" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="261" spans="2:2">
       <c r="B261" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="262" spans="2:2">
       <c r="B262" t="s">
-        <v>676</v>
+        <v>460</v>
       </c>
     </row>
     <row r="263" spans="2:2">
       <c r="B263" t="s">
-        <v>462</v>
+        <v>676</v>
       </c>
     </row>
     <row r="264" spans="2:2">
       <c r="B264" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="265" spans="2:2">
       <c r="B265" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="266" spans="2:2">
       <c r="B266" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="267" spans="2:2">
       <c r="B267" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="268" spans="2:2">
       <c r="B268" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="269" spans="2:2">
       <c r="B269" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="270" spans="2:2">
       <c r="B270" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="271" spans="2:2">
       <c r="B271" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="272" spans="2:2">
       <c r="B272" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="273" spans="2:2">
       <c r="B273" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="274" spans="2:2">
       <c r="B274" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="275" spans="2:2">
       <c r="B275" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="276" spans="2:2">
       <c r="B276" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="277" spans="2:2">
       <c r="B277" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="278" spans="2:2">
       <c r="B278" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="279" spans="2:2">
       <c r="B279" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="280" spans="2:2">
       <c r="B280" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="281" spans="2:2">
       <c r="B281" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="282" spans="2:2">
       <c r="B282" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="283" spans="2:2">
       <c r="B283" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="284" spans="2:2">
       <c r="B284" t="s">
-        <v>740</v>
+        <v>503</v>
       </c>
     </row>
     <row r="285" spans="2:2">
       <c r="B285" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="286" spans="2:2">
       <c r="B286" t="s">
-        <v>505</v>
+        <v>747</v>
       </c>
     </row>
     <row r="287" spans="2:2">
       <c r="B287" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="288" spans="2:2">
       <c r="B288" t="s">
-        <v>746</v>
+        <v>507</v>
       </c>
     </row>
     <row r="289" spans="2:2">
       <c r="B289" t="s">
-        <v>679</v>
+        <v>749</v>
       </c>
     </row>
     <row r="290" spans="2:2">
       <c r="B290" t="s">
-        <v>509</v>
+        <v>679</v>
       </c>
     </row>
     <row r="291" spans="2:2">
       <c r="B291" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
     <row r="292" spans="2:2">
       <c r="B292" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="293" spans="2:2">
       <c r="B293" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="294" spans="2:2">
       <c r="B294" t="s">
-        <v>699</v>
+        <v>515</v>
       </c>
     </row>
     <row r="295" spans="2:2">
       <c r="B295" t="s">
-        <v>517</v>
+        <v>702</v>
       </c>
     </row>
     <row r="296" spans="2:2">
       <c r="B296" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="297" spans="2:2">
       <c r="B297" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="298" spans="2:2">
       <c r="B298" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="299" spans="2:2">
       <c r="B299" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="300" spans="2:2">
       <c r="B300" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="301" spans="2:2">
       <c r="B301" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="302" spans="2:2">
       <c r="B302" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="303" spans="2:2">
       <c r="B303" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="304" spans="2:2">
       <c r="B304" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
     </row>
     <row r="305" spans="2:2">
       <c r="B305" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="306" spans="2:2">
       <c r="B306" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="307" spans="2:2">
       <c r="B307" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="308" spans="2:2">
       <c r="B308" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="309" spans="2:2">
       <c r="B309" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
     <row r="310" spans="2:2">
       <c r="B310" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
     </row>
     <row r="311" spans="2:2">
       <c r="B311" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="312" spans="2:2">
       <c r="B312" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="313" spans="2:2">
       <c r="B313" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="314" spans="2:2">
       <c r="B314" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
     </row>
     <row r="315" spans="2:2">
       <c r="B315" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="316" spans="2:2">
       <c r="B316" t="s">
-        <v>682</v>
+        <v>557</v>
       </c>
     </row>
     <row r="317" spans="2:2">
       <c r="B317" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="318" spans="2:2">
       <c r="B318" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
     </row>
     <row r="319" spans="2:2">
       <c r="B319" t="s">
-        <v>559</v>
+        <v>687</v>
       </c>
     </row>
     <row r="320" spans="2:2">
       <c r="B320" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
     <row r="321" spans="2:2">
       <c r="B321" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="322" spans="2:2">
       <c r="B322" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="323" spans="2:2">
       <c r="B323" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="324" spans="2:2">
       <c r="B324" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="325" spans="2:2">
       <c r="B325" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="326" spans="2:2">
       <c r="B326" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="327" spans="2:2">
       <c r="B327" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="328" spans="2:2">
       <c r="B328" t="s">
-        <v>726</v>
+        <v>575</v>
       </c>
     </row>
     <row r="329" spans="2:2">
       <c r="B329" t="s">
-        <v>577</v>
+        <v>729</v>
       </c>
     </row>
     <row r="330" spans="2:2">
       <c r="B330" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
     </row>
     <row r="331" spans="2:2">
       <c r="B331" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="332" spans="2:2">
       <c r="B332" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="333" spans="2:2">
       <c r="B333" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
     </row>
     <row r="334" spans="2:2">
       <c r="B334" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
     </row>
     <row r="335" spans="2:2">
       <c r="B335" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="336" spans="2:2">
       <c r="B336" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="337" spans="1:2">
       <c r="B337" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="338" spans="1:2">
       <c r="B338" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
     </row>
     <row r="339" spans="1:2">
       <c r="B339" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="340" spans="1:2">
+      <c r="B340" t="s">
         <v>598</v>
       </c>
     </row>
-    <row r="341" spans="1:2">
-      <c r="A341" t="s">
-        <v>752</v>
-      </c>
-      <c r="B341" t="s">
+    <row r="342" spans="1:2">
+      <c r="A342" t="s">
+        <v>755</v>
+      </c>
+      <c r="B342" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="343" spans="1:2">
-      <c r="A343" t="s">
-        <v>753</v>
-      </c>
-      <c r="B343" t="s">
+    <row r="344" spans="1:2">
+      <c r="A344" t="s">
+        <v>756</v>
+      </c>
+      <c r="B344" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="344" spans="1:2">
-      <c r="B344" t="s">
+    <row r="345" spans="1:2">
+      <c r="B345" t="s">
         <v>676</v>
       </c>
     </row>
-    <row r="346" spans="1:2">
-      <c r="A346" t="s">
-        <v>754</v>
-      </c>
-      <c r="B346" t="s">
+    <row r="347" spans="1:2">
+      <c r="A347" t="s">
+        <v>757</v>
+      </c>
+      <c r="B347" t="s">
         <v>619</v>
-      </c>
-    </row>
-    <row r="347" spans="1:2">
-      <c r="B347" t="s">
-        <v>719</v>
       </c>
     </row>
     <row r="348" spans="1:2">
       <c r="B348" t="s">
-        <v>633</v>
+        <v>722</v>
       </c>
     </row>
     <row r="349" spans="1:2">
       <c r="B349" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="350" spans="1:2">
+      <c r="B350" t="s">
         <v>644</v>
       </c>
     </row>
@@ -10039,7 +10053,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="110.7109375" customWidth="1"/>
@@ -10125,7 +10139,7 @@
         <v>699</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>2.66</v>
       </c>
       <c r="C6" t="s">
         <v>700</v>
@@ -10134,6 +10148,23 @@
         <v>8</v>
       </c>
       <c r="E6" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>702</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>703</v>
+      </c>
+      <c r="D7" t="s">
+        <v>8</v>
+      </c>
+      <c r="E7" t="s">
         <v>643</v>
       </c>
     </row>
@@ -10154,7 +10185,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10176,19 +10207,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="B3">
         <v>2.2</v>
       </c>
       <c r="C3" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
     </row>
   </sheetData>
@@ -10208,7 +10239,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10230,19 +10261,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B3">
         <v>1.32</v>
       </c>
       <c r="C3" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
     </row>
   </sheetData>
@@ -10262,7 +10293,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10284,19 +10315,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="B3">
         <v>2.45</v>
       </c>
       <c r="C3" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
     </row>
   </sheetData>
@@ -10316,7 +10347,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10338,47 +10369,47 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="B3">
         <v>1.9</v>
       </c>
       <c r="C3" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
       <c r="B4">
         <v>2.11</v>
       </c>
       <c r="C4" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="B5">
         <v>2.7</v>
       </c>
       <c r="C5" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -10389,13 +10420,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="B6">
         <v>2.58</v>
       </c>
       <c r="C6" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -10406,30 +10437,30 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="B7">
         <v>1.93</v>
       </c>
       <c r="C7" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="B8">
         <v>2.05</v>
       </c>
       <c r="C8" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
@@ -10455,7 +10486,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10477,13 +10508,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="B3">
         <v>0.93</v>
       </c>
       <c r="C3" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -10509,7 +10540,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10531,19 +10562,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="B3">
         <v>2.17</v>
       </c>
       <c r="C3" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
weekly update, 2022-03-16, SARS-CoV-2
</commit_message>
<xml_diff>
--- a/pdb/nsp3/SARS-CoV-2/domains_and_infos_of_nsp3.xlsx
+++ b/pdb/nsp3/SARS-CoV-2/domains_and_infos_of_nsp3.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1776" uniqueCount="758">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1801" uniqueCount="769">
   <si>
     <t>nsp3_Macro1_</t>
   </si>
@@ -2125,6 +2125,15 @@
     <t>2020-04-28</t>
   </si>
   <si>
+    <t>7qch</t>
+  </si>
+  <si>
+    <t>STRUCTURE OF SARS-COV-2 PAPAIN-LIKE PROTEASE BOUND TO N-(3,5- DIMETHOXY-4-HYDROXYBENZYLIDEN)THIOSEMICARBAZONE</t>
+  </si>
+  <si>
+    <t>2021-11-24</t>
+  </si>
+  <si>
     <t>7tzj</t>
   </si>
   <si>
@@ -2134,10 +2143,34 @@
     <t>2022-02-15</t>
   </si>
   <si>
+    <t>7qci</t>
+  </si>
+  <si>
+    <t>STRUCTURE OF SARS-COV-2 PAPAIN-LIKE PROTEASE BOUND TO N-(3,4- DIHYDROXYBENZYLIDENE)-THIOSEMICARBAZONE</t>
+  </si>
+  <si>
+    <t>7qcj</t>
+  </si>
+  <si>
+    <t>STRUCTURE OF SARS-COV-2 PAPAIN-LIKE PROTEASE BOUND TO N-(2,4- DIHYDROXYBENZYLIDENE)-THIOSEMICARBAZONE</t>
+  </si>
+  <si>
     <t>7sgv</t>
   </si>
   <si>
     <t>PAPAIN-LIKE PROTEASE OF SARS COV-2, C111S MUTANT, IN COMPLEX WITH PLP_SNYDER630 INHIBITOR</t>
+  </si>
+  <si>
+    <t>7qck</t>
+  </si>
+  <si>
+    <t>STRUCTURE OF SARS-COV-2 PAPAIN-LIKE PROTEASE BOUND TO N-(2,5- DIHYDROXYBENZYLIDENE)-THIOSEMICARBAZONE</t>
+  </si>
+  <si>
+    <t>7qcm</t>
+  </si>
+  <si>
+    <t>STRUCTURE OF SARS-COV-2 PAPAIN-LIKE PROTEASE BOUND TO N-(3-METHOXY-4- HYDROXY-ACETOPHENONE)THIOSEMICARBAZONE</t>
   </si>
   <si>
     <t>nsp3_betaSM-M_</t>
@@ -7540,7 +7573,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>738</v>
+        <v>749</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7562,19 +7595,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>739</v>
+        <v>750</v>
       </c>
       <c r="B3">
         <v>2.72</v>
       </c>
       <c r="C3" t="s">
-        <v>740</v>
+        <v>751</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>741</v>
+        <v>752</v>
       </c>
     </row>
   </sheetData>
@@ -7594,7 +7627,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>742</v>
+        <v>753</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7616,19 +7649,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>743</v>
+        <v>754</v>
       </c>
       <c r="B3">
         <v>2.68</v>
       </c>
       <c r="C3" t="s">
-        <v>744</v>
+        <v>755</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>745</v>
+        <v>756</v>
       </c>
     </row>
   </sheetData>
@@ -7648,7 +7681,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>746</v>
+        <v>757</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7670,13 +7703,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>747</v>
+        <v>758</v>
       </c>
       <c r="B3">
         <v>3.21</v>
       </c>
       <c r="C3" t="s">
-        <v>748</v>
+        <v>759</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -7687,19 +7720,19 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>749</v>
+        <v>760</v>
       </c>
       <c r="B4">
         <v>2.73</v>
       </c>
       <c r="C4" t="s">
-        <v>750</v>
+        <v>761</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>751</v>
+        <v>762</v>
       </c>
     </row>
   </sheetData>
@@ -7709,7 +7742,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B350"/>
+  <dimension ref="A1:B355"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
@@ -7717,12 +7750,12 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>752</v>
+        <v>763</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>753</v>
+        <v>764</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -7730,7 +7763,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>754</v>
+        <v>765</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -7893,7 +7926,7 @@
     </row>
     <row r="35" spans="2:2">
       <c r="B35" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
     </row>
     <row r="36" spans="2:2">
@@ -7918,7 +7951,7 @@
     </row>
     <row r="40" spans="2:2">
       <c r="B40" t="s">
-        <v>709</v>
+        <v>720</v>
       </c>
     </row>
     <row r="41" spans="2:2">
@@ -7943,7 +7976,7 @@
     </row>
     <row r="45" spans="2:2">
       <c r="B45" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
     </row>
     <row r="46" spans="2:2">
@@ -7993,7 +8026,7 @@
     </row>
     <row r="55" spans="2:2">
       <c r="B55" t="s">
-        <v>717</v>
+        <v>728</v>
       </c>
     </row>
     <row r="56" spans="2:2">
@@ -8223,7 +8256,7 @@
     </row>
     <row r="101" spans="2:2">
       <c r="B101" t="s">
-        <v>720</v>
+        <v>731</v>
       </c>
     </row>
     <row r="102" spans="2:2">
@@ -8353,7 +8386,7 @@
     </row>
     <row r="127" spans="2:2">
       <c r="B127" t="s">
-        <v>732</v>
+        <v>743</v>
       </c>
     </row>
     <row r="128" spans="2:2">
@@ -8363,7 +8396,7 @@
     </row>
     <row r="129" spans="2:2">
       <c r="B129" t="s">
-        <v>722</v>
+        <v>733</v>
       </c>
     </row>
     <row r="130" spans="2:2">
@@ -8468,7 +8501,7 @@
     </row>
     <row r="150" spans="2:2">
       <c r="B150" t="s">
-        <v>724</v>
+        <v>735</v>
       </c>
     </row>
     <row r="151" spans="2:2">
@@ -8478,990 +8511,1015 @@
     </row>
     <row r="152" spans="2:2">
       <c r="B152" t="s">
-        <v>277</v>
+        <v>699</v>
       </c>
     </row>
     <row r="153" spans="2:2">
       <c r="B153" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="154" spans="2:2">
       <c r="B154" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="155" spans="2:2">
       <c r="B155" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="156" spans="2:2">
       <c r="B156" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="157" spans="2:2">
       <c r="B157" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="158" spans="2:2">
       <c r="B158" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="159" spans="2:2">
       <c r="B159" t="s">
-        <v>636</v>
+        <v>290</v>
       </c>
     </row>
     <row r="160" spans="2:2">
       <c r="B160" t="s">
-        <v>292</v>
+        <v>636</v>
       </c>
     </row>
     <row r="161" spans="2:2">
       <c r="B161" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="162" spans="2:2">
       <c r="B162" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="163" spans="2:2">
       <c r="B163" t="s">
-        <v>638</v>
+        <v>296</v>
       </c>
     </row>
     <row r="164" spans="2:2">
       <c r="B164" t="s">
-        <v>298</v>
+        <v>638</v>
       </c>
     </row>
     <row r="165" spans="2:2">
       <c r="B165" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="166" spans="2:2">
       <c r="B166" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="167" spans="2:2">
       <c r="B167" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="168" spans="2:2">
       <c r="B168" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="169" spans="2:2">
       <c r="B169" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="170" spans="2:2">
       <c r="B170" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="171" spans="2:2">
       <c r="B171" t="s">
-        <v>641</v>
+        <v>310</v>
       </c>
     </row>
     <row r="172" spans="2:2">
       <c r="B172" t="s">
-        <v>312</v>
+        <v>641</v>
       </c>
     </row>
     <row r="173" spans="2:2">
       <c r="B173" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="174" spans="2:2">
       <c r="B174" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="175" spans="2:2">
       <c r="B175" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="176" spans="2:2">
       <c r="B176" t="s">
-        <v>735</v>
+        <v>318</v>
       </c>
     </row>
     <row r="177" spans="2:2">
       <c r="B177" t="s">
-        <v>320</v>
+        <v>746</v>
       </c>
     </row>
     <row r="178" spans="2:2">
       <c r="B178" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="179" spans="2:2">
       <c r="B179" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="180" spans="2:2">
       <c r="B180" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="181" spans="2:2">
       <c r="B181" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="182" spans="2:2">
       <c r="B182" t="s">
-        <v>644</v>
+        <v>328</v>
       </c>
     </row>
     <row r="183" spans="2:2">
       <c r="B183" t="s">
-        <v>330</v>
+        <v>644</v>
       </c>
     </row>
     <row r="184" spans="2:2">
       <c r="B184" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="185" spans="2:2">
       <c r="B185" t="s">
-        <v>646</v>
+        <v>332</v>
       </c>
     </row>
     <row r="186" spans="2:2">
       <c r="B186" t="s">
-        <v>333</v>
+        <v>646</v>
       </c>
     </row>
     <row r="187" spans="2:2">
       <c r="B187" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="188" spans="2:2">
       <c r="B188" t="s">
-        <v>699</v>
+        <v>335</v>
       </c>
     </row>
     <row r="189" spans="2:2">
       <c r="B189" t="s">
-        <v>649</v>
+        <v>702</v>
       </c>
     </row>
     <row r="190" spans="2:2">
       <c r="B190" t="s">
-        <v>337</v>
+        <v>649</v>
       </c>
     </row>
     <row r="191" spans="2:2">
       <c r="B191" t="s">
-        <v>652</v>
+        <v>337</v>
       </c>
     </row>
     <row r="192" spans="2:2">
       <c r="B192" t="s">
-        <v>338</v>
+        <v>652</v>
       </c>
     </row>
     <row r="193" spans="2:2">
       <c r="B193" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="194" spans="2:2">
       <c r="B194" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="195" spans="2:2">
       <c r="B195" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="196" spans="2:2">
       <c r="B196" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="197" spans="2:2">
       <c r="B197" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="198" spans="2:2">
       <c r="B198" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="199" spans="2:2">
       <c r="B199" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
     </row>
     <row r="200" spans="2:2">
       <c r="B200" t="s">
-        <v>355</v>
+        <v>705</v>
       </c>
     </row>
     <row r="201" spans="2:2">
       <c r="B201" t="s">
-        <v>357</v>
+        <v>353</v>
       </c>
     </row>
     <row r="202" spans="2:2">
       <c r="B202" t="s">
-        <v>359</v>
+        <v>355</v>
       </c>
     </row>
     <row r="203" spans="2:2">
       <c r="B203" t="s">
-        <v>361</v>
+        <v>357</v>
       </c>
     </row>
     <row r="204" spans="2:2">
       <c r="B204" t="s">
-        <v>654</v>
+        <v>359</v>
       </c>
     </row>
     <row r="205" spans="2:2">
       <c r="B205" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
     </row>
     <row r="206" spans="2:2">
       <c r="B206" t="s">
-        <v>365</v>
+        <v>654</v>
       </c>
     </row>
     <row r="207" spans="2:2">
       <c r="B207" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
     </row>
     <row r="208" spans="2:2">
       <c r="B208" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
     </row>
     <row r="209" spans="2:2">
       <c r="B209" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
     </row>
     <row r="210" spans="2:2">
       <c r="B210" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
     </row>
     <row r="211" spans="2:2">
       <c r="B211" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="212" spans="2:2">
       <c r="B212" t="s">
-        <v>657</v>
+        <v>373</v>
       </c>
     </row>
     <row r="213" spans="2:2">
       <c r="B213" t="s">
-        <v>660</v>
+        <v>374</v>
       </c>
     </row>
     <row r="214" spans="2:2">
       <c r="B214" t="s">
-        <v>377</v>
+        <v>657</v>
       </c>
     </row>
     <row r="215" spans="2:2">
       <c r="B215" t="s">
-        <v>379</v>
+        <v>660</v>
       </c>
     </row>
     <row r="216" spans="2:2">
       <c r="B216" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="217" spans="2:2">
       <c r="B217" t="s">
-        <v>726</v>
+        <v>379</v>
       </c>
     </row>
     <row r="218" spans="2:2">
       <c r="B218" t="s">
-        <v>382</v>
+        <v>380</v>
       </c>
     </row>
     <row r="219" spans="2:2">
       <c r="B219" t="s">
-        <v>739</v>
+        <v>737</v>
       </c>
     </row>
     <row r="220" spans="2:2">
       <c r="B220" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="221" spans="2:2">
       <c r="B221" t="s">
-        <v>386</v>
+        <v>750</v>
       </c>
     </row>
     <row r="222" spans="2:2">
       <c r="B222" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
     </row>
     <row r="223" spans="2:2">
       <c r="B223" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
     </row>
     <row r="224" spans="2:2">
       <c r="B224" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="225" spans="2:2">
       <c r="B225" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="226" spans="2:2">
       <c r="B226" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
     </row>
     <row r="227" spans="2:2">
       <c r="B227" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
     </row>
     <row r="228" spans="2:2">
       <c r="B228" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
     <row r="229" spans="2:2">
       <c r="B229" t="s">
-        <v>663</v>
+        <v>398</v>
       </c>
     </row>
     <row r="230" spans="2:2">
       <c r="B230" t="s">
-        <v>666</v>
+        <v>400</v>
       </c>
     </row>
     <row r="231" spans="2:2">
       <c r="B231" t="s">
-        <v>402</v>
+        <v>663</v>
       </c>
     </row>
     <row r="232" spans="2:2">
       <c r="B232" t="s">
-        <v>404</v>
+        <v>666</v>
       </c>
     </row>
     <row r="233" spans="2:2">
       <c r="B233" t="s">
-        <v>407</v>
+        <v>402</v>
       </c>
     </row>
     <row r="234" spans="2:2">
       <c r="B234" t="s">
-        <v>409</v>
+        <v>404</v>
       </c>
     </row>
     <row r="235" spans="2:2">
       <c r="B235" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
     </row>
     <row r="236" spans="2:2">
       <c r="B236" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
     </row>
     <row r="237" spans="2:2">
       <c r="B237" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
     </row>
     <row r="238" spans="2:2">
       <c r="B238" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
     </row>
     <row r="239" spans="2:2">
       <c r="B239" t="s">
-        <v>420</v>
+        <v>415</v>
       </c>
     </row>
     <row r="240" spans="2:2">
       <c r="B240" t="s">
-        <v>669</v>
+        <v>417</v>
       </c>
     </row>
     <row r="241" spans="2:2">
       <c r="B241" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="242" spans="2:2">
       <c r="B242" t="s">
-        <v>423</v>
+        <v>707</v>
       </c>
     </row>
     <row r="243" spans="2:2">
       <c r="B243" t="s">
-        <v>425</v>
+        <v>669</v>
       </c>
     </row>
     <row r="244" spans="2:2">
       <c r="B244" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
     </row>
     <row r="245" spans="2:2">
       <c r="B245" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
     </row>
     <row r="246" spans="2:2">
       <c r="B246" t="s">
-        <v>671</v>
+        <v>425</v>
       </c>
     </row>
     <row r="247" spans="2:2">
       <c r="B247" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
     </row>
     <row r="248" spans="2:2">
       <c r="B248" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
     </row>
     <row r="249" spans="2:2">
       <c r="B249" t="s">
-        <v>435</v>
+        <v>671</v>
       </c>
     </row>
     <row r="250" spans="2:2">
       <c r="B250" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
     </row>
     <row r="251" spans="2:2">
       <c r="B251" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
     </row>
     <row r="252" spans="2:2">
       <c r="B252" t="s">
-        <v>441</v>
+        <v>435</v>
       </c>
     </row>
     <row r="253" spans="2:2">
       <c r="B253" t="s">
-        <v>444</v>
+        <v>437</v>
       </c>
     </row>
     <row r="254" spans="2:2">
       <c r="B254" t="s">
-        <v>446</v>
+        <v>439</v>
       </c>
     </row>
     <row r="255" spans="2:2">
       <c r="B255" t="s">
-        <v>448</v>
+        <v>441</v>
       </c>
     </row>
     <row r="256" spans="2:2">
       <c r="B256" t="s">
-        <v>450</v>
+        <v>444</v>
       </c>
     </row>
     <row r="257" spans="2:2">
       <c r="B257" t="s">
-        <v>673</v>
+        <v>446</v>
       </c>
     </row>
     <row r="258" spans="2:2">
       <c r="B258" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
     </row>
     <row r="259" spans="2:2">
       <c r="B259" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
     </row>
     <row r="260" spans="2:2">
       <c r="B260" t="s">
-        <v>456</v>
+        <v>673</v>
       </c>
     </row>
     <row r="261" spans="2:2">
       <c r="B261" t="s">
-        <v>458</v>
+        <v>452</v>
       </c>
     </row>
     <row r="262" spans="2:2">
       <c r="B262" t="s">
-        <v>460</v>
+        <v>454</v>
       </c>
     </row>
     <row r="263" spans="2:2">
       <c r="B263" t="s">
-        <v>676</v>
+        <v>456</v>
       </c>
     </row>
     <row r="264" spans="2:2">
       <c r="B264" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
     </row>
     <row r="265" spans="2:2">
       <c r="B265" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="266" spans="2:2">
       <c r="B266" t="s">
-        <v>465</v>
+        <v>676</v>
       </c>
     </row>
     <row r="267" spans="2:2">
       <c r="B267" t="s">
-        <v>467</v>
+        <v>462</v>
       </c>
     </row>
     <row r="268" spans="2:2">
       <c r="B268" t="s">
-        <v>469</v>
+        <v>463</v>
       </c>
     </row>
     <row r="269" spans="2:2">
       <c r="B269" t="s">
-        <v>471</v>
+        <v>465</v>
       </c>
     </row>
     <row r="270" spans="2:2">
       <c r="B270" t="s">
-        <v>473</v>
+        <v>467</v>
       </c>
     </row>
     <row r="271" spans="2:2">
       <c r="B271" t="s">
-        <v>475</v>
+        <v>469</v>
       </c>
     </row>
     <row r="272" spans="2:2">
       <c r="B272" t="s">
-        <v>477</v>
+        <v>471</v>
       </c>
     </row>
     <row r="273" spans="2:2">
       <c r="B273" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
     </row>
     <row r="274" spans="2:2">
       <c r="B274" t="s">
-        <v>481</v>
+        <v>475</v>
       </c>
     </row>
     <row r="275" spans="2:2">
       <c r="B275" t="s">
-        <v>483</v>
+        <v>477</v>
       </c>
     </row>
     <row r="276" spans="2:2">
       <c r="B276" t="s">
-        <v>485</v>
+        <v>479</v>
       </c>
     </row>
     <row r="277" spans="2:2">
       <c r="B277" t="s">
-        <v>487</v>
+        <v>481</v>
       </c>
     </row>
     <row r="278" spans="2:2">
       <c r="B278" t="s">
-        <v>489</v>
+        <v>483</v>
       </c>
     </row>
     <row r="279" spans="2:2">
       <c r="B279" t="s">
-        <v>491</v>
+        <v>485</v>
       </c>
     </row>
     <row r="280" spans="2:2">
       <c r="B280" t="s">
-        <v>493</v>
+        <v>487</v>
       </c>
     </row>
     <row r="281" spans="2:2">
       <c r="B281" t="s">
-        <v>495</v>
+        <v>489</v>
       </c>
     </row>
     <row r="282" spans="2:2">
       <c r="B282" t="s">
-        <v>498</v>
+        <v>491</v>
       </c>
     </row>
     <row r="283" spans="2:2">
       <c r="B283" t="s">
-        <v>500</v>
+        <v>493</v>
       </c>
     </row>
     <row r="284" spans="2:2">
       <c r="B284" t="s">
-        <v>503</v>
+        <v>495</v>
       </c>
     </row>
     <row r="285" spans="2:2">
       <c r="B285" t="s">
-        <v>743</v>
+        <v>498</v>
       </c>
     </row>
     <row r="286" spans="2:2">
       <c r="B286" t="s">
-        <v>747</v>
+        <v>500</v>
       </c>
     </row>
     <row r="287" spans="2:2">
       <c r="B287" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="288" spans="2:2">
       <c r="B288" t="s">
-        <v>507</v>
+        <v>754</v>
       </c>
     </row>
     <row r="289" spans="2:2">
       <c r="B289" t="s">
-        <v>749</v>
+        <v>758</v>
       </c>
     </row>
     <row r="290" spans="2:2">
       <c r="B290" t="s">
-        <v>679</v>
+        <v>505</v>
       </c>
     </row>
     <row r="291" spans="2:2">
       <c r="B291" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="292" spans="2:2">
       <c r="B292" t="s">
-        <v>511</v>
+        <v>760</v>
       </c>
     </row>
     <row r="293" spans="2:2">
       <c r="B293" t="s">
-        <v>513</v>
+        <v>679</v>
       </c>
     </row>
     <row r="294" spans="2:2">
       <c r="B294" t="s">
-        <v>515</v>
+        <v>509</v>
       </c>
     </row>
     <row r="295" spans="2:2">
       <c r="B295" t="s">
-        <v>702</v>
+        <v>511</v>
       </c>
     </row>
     <row r="296" spans="2:2">
       <c r="B296" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
     </row>
     <row r="297" spans="2:2">
       <c r="B297" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
     </row>
     <row r="298" spans="2:2">
       <c r="B298" t="s">
-        <v>521</v>
+        <v>709</v>
       </c>
     </row>
     <row r="299" spans="2:2">
       <c r="B299" t="s">
-        <v>523</v>
+        <v>517</v>
       </c>
     </row>
     <row r="300" spans="2:2">
       <c r="B300" t="s">
-        <v>525</v>
+        <v>519</v>
       </c>
     </row>
     <row r="301" spans="2:2">
       <c r="B301" t="s">
-        <v>527</v>
+        <v>521</v>
       </c>
     </row>
     <row r="302" spans="2:2">
       <c r="B302" t="s">
-        <v>529</v>
+        <v>711</v>
       </c>
     </row>
     <row r="303" spans="2:2">
       <c r="B303" t="s">
-        <v>531</v>
+        <v>523</v>
       </c>
     </row>
     <row r="304" spans="2:2">
       <c r="B304" t="s">
-        <v>533</v>
+        <v>525</v>
       </c>
     </row>
     <row r="305" spans="2:2">
       <c r="B305" t="s">
-        <v>535</v>
+        <v>527</v>
       </c>
     </row>
     <row r="306" spans="2:2">
       <c r="B306" t="s">
-        <v>537</v>
+        <v>529</v>
       </c>
     </row>
     <row r="307" spans="2:2">
       <c r="B307" t="s">
-        <v>539</v>
+        <v>531</v>
       </c>
     </row>
     <row r="308" spans="2:2">
       <c r="B308" t="s">
-        <v>541</v>
+        <v>533</v>
       </c>
     </row>
     <row r="309" spans="2:2">
       <c r="B309" t="s">
-        <v>543</v>
+        <v>713</v>
       </c>
     </row>
     <row r="310" spans="2:2">
       <c r="B310" t="s">
-        <v>545</v>
+        <v>535</v>
       </c>
     </row>
     <row r="311" spans="2:2">
       <c r="B311" t="s">
-        <v>547</v>
+        <v>537</v>
       </c>
     </row>
     <row r="312" spans="2:2">
       <c r="B312" t="s">
-        <v>549</v>
+        <v>539</v>
       </c>
     </row>
     <row r="313" spans="2:2">
       <c r="B313" t="s">
-        <v>551</v>
+        <v>541</v>
       </c>
     </row>
     <row r="314" spans="2:2">
       <c r="B314" t="s">
-        <v>553</v>
+        <v>543</v>
       </c>
     </row>
     <row r="315" spans="2:2">
       <c r="B315" t="s">
-        <v>555</v>
+        <v>545</v>
       </c>
     </row>
     <row r="316" spans="2:2">
       <c r="B316" t="s">
-        <v>557</v>
+        <v>547</v>
       </c>
     </row>
     <row r="317" spans="2:2">
       <c r="B317" t="s">
-        <v>682</v>
+        <v>549</v>
       </c>
     </row>
     <row r="318" spans="2:2">
       <c r="B318" t="s">
-        <v>684</v>
+        <v>551</v>
       </c>
     </row>
     <row r="319" spans="2:2">
       <c r="B319" t="s">
-        <v>687</v>
+        <v>553</v>
       </c>
     </row>
     <row r="320" spans="2:2">
       <c r="B320" t="s">
-        <v>559</v>
+        <v>555</v>
       </c>
     </row>
     <row r="321" spans="2:2">
       <c r="B321" t="s">
-        <v>561</v>
+        <v>557</v>
       </c>
     </row>
     <row r="322" spans="2:2">
       <c r="B322" t="s">
-        <v>563</v>
+        <v>682</v>
       </c>
     </row>
     <row r="323" spans="2:2">
       <c r="B323" t="s">
-        <v>565</v>
+        <v>684</v>
       </c>
     </row>
     <row r="324" spans="2:2">
       <c r="B324" t="s">
-        <v>567</v>
+        <v>687</v>
       </c>
     </row>
     <row r="325" spans="2:2">
       <c r="B325" t="s">
-        <v>569</v>
+        <v>559</v>
       </c>
     </row>
     <row r="326" spans="2:2">
       <c r="B326" t="s">
-        <v>571</v>
+        <v>561</v>
       </c>
     </row>
     <row r="327" spans="2:2">
       <c r="B327" t="s">
-        <v>573</v>
+        <v>563</v>
       </c>
     </row>
     <row r="328" spans="2:2">
       <c r="B328" t="s">
-        <v>575</v>
+        <v>565</v>
       </c>
     </row>
     <row r="329" spans="2:2">
       <c r="B329" t="s">
-        <v>729</v>
+        <v>567</v>
       </c>
     </row>
     <row r="330" spans="2:2">
       <c r="B330" t="s">
-        <v>577</v>
+        <v>569</v>
       </c>
     </row>
     <row r="331" spans="2:2">
       <c r="B331" t="s">
-        <v>579</v>
+        <v>571</v>
       </c>
     </row>
     <row r="332" spans="2:2">
       <c r="B332" t="s">
-        <v>581</v>
+        <v>573</v>
       </c>
     </row>
     <row r="333" spans="2:2">
       <c r="B333" t="s">
-        <v>583</v>
+        <v>575</v>
       </c>
     </row>
     <row r="334" spans="2:2">
       <c r="B334" t="s">
-        <v>585</v>
+        <v>740</v>
       </c>
     </row>
     <row r="335" spans="2:2">
       <c r="B335" t="s">
-        <v>587</v>
+        <v>577</v>
       </c>
     </row>
     <row r="336" spans="2:2">
       <c r="B336" t="s">
-        <v>589</v>
+        <v>579</v>
       </c>
     </row>
     <row r="337" spans="1:2">
       <c r="B337" t="s">
-        <v>591</v>
+        <v>581</v>
       </c>
     </row>
     <row r="338" spans="1:2">
       <c r="B338" t="s">
-        <v>593</v>
+        <v>583</v>
       </c>
     </row>
     <row r="339" spans="1:2">
       <c r="B339" t="s">
-        <v>596</v>
+        <v>585</v>
       </c>
     </row>
     <row r="340" spans="1:2">
       <c r="B340" t="s">
-        <v>598</v>
+        <v>587</v>
+      </c>
+    </row>
+    <row r="341" spans="1:2">
+      <c r="B341" t="s">
+        <v>589</v>
       </c>
     </row>
     <row r="342" spans="1:2">
-      <c r="A342" t="s">
-        <v>755</v>
-      </c>
       <c r="B342" t="s">
-        <v>696</v>
+        <v>591</v>
+      </c>
+    </row>
+    <row r="343" spans="1:2">
+      <c r="B343" t="s">
+        <v>593</v>
       </c>
     </row>
     <row r="344" spans="1:2">
-      <c r="A344" t="s">
-        <v>756</v>
-      </c>
       <c r="B344" t="s">
-        <v>616</v>
+        <v>596</v>
       </c>
     </row>
     <row r="345" spans="1:2">
       <c r="B345" t="s">
-        <v>676</v>
+        <v>598</v>
       </c>
     </row>
     <row r="347" spans="1:2">
       <c r="A347" t="s">
-        <v>757</v>
+        <v>766</v>
       </c>
       <c r="B347" t="s">
-        <v>619</v>
-      </c>
-    </row>
-    <row r="348" spans="1:2">
-      <c r="B348" t="s">
-        <v>722</v>
+        <v>696</v>
       </c>
     </row>
     <row r="349" spans="1:2">
+      <c r="A349" t="s">
+        <v>767</v>
+      </c>
       <c r="B349" t="s">
-        <v>633</v>
+        <v>616</v>
       </c>
     </row>
     <row r="350" spans="1:2">
       <c r="B350" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2">
+      <c r="A352" t="s">
+        <v>768</v>
+      </c>
+      <c r="B352" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="353" spans="2:2">
+      <c r="B353" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="354" spans="2:2">
+      <c r="B354" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="355" spans="2:2">
+      <c r="B355" t="s">
         <v>644</v>
       </c>
     </row>
@@ -10053,7 +10111,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="110.7109375" customWidth="1"/>
@@ -10139,7 +10197,7 @@
         <v>699</v>
       </c>
       <c r="B6">
-        <v>2.66</v>
+        <v>1.88</v>
       </c>
       <c r="C6" t="s">
         <v>700</v>
@@ -10156,7 +10214,7 @@
         <v>702</v>
       </c>
       <c r="B7">
-        <v>2</v>
+        <v>2.66</v>
       </c>
       <c r="C7" t="s">
         <v>703</v>
@@ -10165,7 +10223,92 @@
         <v>8</v>
       </c>
       <c r="E7" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>705</v>
+      </c>
+      <c r="B8">
+        <v>1.76</v>
+      </c>
+      <c r="C8" t="s">
+        <v>706</v>
+      </c>
+      <c r="D8" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>707</v>
+      </c>
+      <c r="B9">
+        <v>1.84</v>
+      </c>
+      <c r="C9" t="s">
+        <v>708</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>709</v>
+      </c>
+      <c r="B10">
+        <v>2</v>
+      </c>
+      <c r="C10" t="s">
+        <v>710</v>
+      </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" t="s">
         <v>643</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>711</v>
+      </c>
+      <c r="B11">
+        <v>1.92</v>
+      </c>
+      <c r="C11" t="s">
+        <v>712</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>713</v>
+      </c>
+      <c r="B12">
+        <v>1.77</v>
+      </c>
+      <c r="C12" t="s">
+        <v>714</v>
+      </c>
+      <c r="D12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" t="s">
+        <v>701</v>
       </c>
     </row>
   </sheetData>
@@ -10185,7 +10328,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>704</v>
+        <v>715</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10207,19 +10350,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>705</v>
+        <v>716</v>
       </c>
       <c r="B3">
         <v>2.2</v>
       </c>
       <c r="C3" t="s">
-        <v>706</v>
+        <v>717</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>707</v>
+        <v>718</v>
       </c>
     </row>
   </sheetData>
@@ -10239,7 +10382,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>708</v>
+        <v>719</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10261,19 +10404,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>709</v>
+        <v>720</v>
       </c>
       <c r="B3">
         <v>1.32</v>
       </c>
       <c r="C3" t="s">
-        <v>710</v>
+        <v>721</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>711</v>
+        <v>722</v>
       </c>
     </row>
   </sheetData>
@@ -10293,7 +10436,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>712</v>
+        <v>723</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10315,19 +10458,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>713</v>
+        <v>724</v>
       </c>
       <c r="B3">
         <v>2.45</v>
       </c>
       <c r="C3" t="s">
-        <v>714</v>
+        <v>725</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>715</v>
+        <v>726</v>
       </c>
     </row>
   </sheetData>
@@ -10347,7 +10490,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>716</v>
+        <v>727</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10369,47 +10512,47 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>717</v>
+        <v>728</v>
       </c>
       <c r="B3">
         <v>1.9</v>
       </c>
       <c r="C3" t="s">
-        <v>718</v>
+        <v>729</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>719</v>
+        <v>730</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>720</v>
+        <v>731</v>
       </c>
       <c r="B4">
         <v>2.11</v>
       </c>
       <c r="C4" t="s">
-        <v>721</v>
+        <v>732</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>719</v>
+        <v>730</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>722</v>
+        <v>733</v>
       </c>
       <c r="B5">
         <v>2.7</v>
       </c>
       <c r="C5" t="s">
-        <v>723</v>
+        <v>734</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -10420,13 +10563,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>724</v>
+        <v>735</v>
       </c>
       <c r="B6">
         <v>2.58</v>
       </c>
       <c r="C6" t="s">
-        <v>725</v>
+        <v>736</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -10437,30 +10580,30 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>726</v>
+        <v>737</v>
       </c>
       <c r="B7">
         <v>1.93</v>
       </c>
       <c r="C7" t="s">
-        <v>727</v>
+        <v>738</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>728</v>
+        <v>739</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>729</v>
+        <v>740</v>
       </c>
       <c r="B8">
         <v>2.05</v>
       </c>
       <c r="C8" t="s">
-        <v>730</v>
+        <v>741</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
@@ -10486,7 +10629,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>731</v>
+        <v>742</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10508,13 +10651,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>732</v>
+        <v>743</v>
       </c>
       <c r="B3">
         <v>0.93</v>
       </c>
       <c r="C3" t="s">
-        <v>733</v>
+        <v>744</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -10540,7 +10683,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>734</v>
+        <v>745</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10562,19 +10705,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>735</v>
+        <v>746</v>
       </c>
       <c r="B3">
         <v>2.17</v>
       </c>
       <c r="C3" t="s">
-        <v>736</v>
+        <v>747</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>737</v>
+        <v>748</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
weekly update, 2022-03-23, SARS-CoV-2
</commit_message>
<xml_diff>
--- a/pdb/nsp3/SARS-CoV-2/domains_and_infos_of_nsp3.xlsx
+++ b/pdb/nsp3/SARS-CoV-2/domains_and_infos_of_nsp3.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1801" uniqueCount="769">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1806" uniqueCount="772">
   <si>
     <t>nsp3_Macro1_</t>
   </si>
@@ -2123,6 +2123,15 @@
   </si>
   <si>
     <t>2020-04-28</t>
+  </si>
+  <si>
+    <t>7qcg</t>
+  </si>
+  <si>
+    <t>STRUCTURE OF SARS-COV-2 PAPAIN-LIKE PROTEASE BOUND TO N-(2- PYRROLIDYL)-3,4,5-TRIHYDROXYBENZOYLHYDRAZONE</t>
+  </si>
+  <si>
+    <t>2021-11-23</t>
   </si>
   <si>
     <t>7qch</t>
@@ -7573,7 +7582,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7595,19 +7604,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="B3">
         <v>2.72</v>
       </c>
       <c r="C3" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
     </row>
   </sheetData>
@@ -7627,7 +7636,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7649,19 +7658,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="B3">
         <v>2.68</v>
       </c>
       <c r="C3" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
     </row>
   </sheetData>
@@ -7681,7 +7690,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7703,13 +7712,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="B3">
         <v>3.21</v>
       </c>
       <c r="C3" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -7720,19 +7729,19 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="B4">
         <v>2.73</v>
       </c>
       <c r="C4" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
     </row>
   </sheetData>
@@ -7742,7 +7751,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B355"/>
+  <dimension ref="A1:B356"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
@@ -7750,12 +7759,12 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>764</v>
+        <v>767</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -7763,7 +7772,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -7926,7 +7935,7 @@
     </row>
     <row r="35" spans="2:2">
       <c r="B35" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
     </row>
     <row r="36" spans="2:2">
@@ -7951,7 +7960,7 @@
     </row>
     <row r="40" spans="2:2">
       <c r="B40" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
     </row>
     <row r="41" spans="2:2">
@@ -7976,7 +7985,7 @@
     </row>
     <row r="45" spans="2:2">
       <c r="B45" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
     </row>
     <row r="46" spans="2:2">
@@ -8026,7 +8035,7 @@
     </row>
     <row r="55" spans="2:2">
       <c r="B55" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
     </row>
     <row r="56" spans="2:2">
@@ -8241,1285 +8250,1290 @@
     </row>
     <row r="98" spans="2:2">
       <c r="B98" t="s">
-        <v>177</v>
+        <v>699</v>
       </c>
     </row>
     <row r="99" spans="2:2">
       <c r="B99" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="100" spans="2:2">
       <c r="B100" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="101" spans="2:2">
       <c r="B101" t="s">
-        <v>731</v>
+        <v>181</v>
       </c>
     </row>
     <row r="102" spans="2:2">
       <c r="B102" t="s">
-        <v>183</v>
+        <v>734</v>
       </c>
     </row>
     <row r="103" spans="2:2">
       <c r="B103" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="104" spans="2:2">
       <c r="B104" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="105" spans="2:2">
       <c r="B105" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="106" spans="2:2">
       <c r="B106" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="107" spans="2:2">
       <c r="B107" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="108" spans="2:2">
       <c r="B108" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="109" spans="2:2">
       <c r="B109" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="110" spans="2:2">
       <c r="B110" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="111" spans="2:2">
       <c r="B111" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="112" spans="2:2">
       <c r="B112" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="113" spans="2:2">
       <c r="B113" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="114" spans="2:2">
       <c r="B114" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="115" spans="2:2">
       <c r="B115" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="116" spans="2:2">
       <c r="B116" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="117" spans="2:2">
       <c r="B117" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="118" spans="2:2">
       <c r="B118" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="119" spans="2:2">
       <c r="B119" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="120" spans="2:2">
       <c r="B120" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="121" spans="2:2">
       <c r="B121" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="122" spans="2:2">
       <c r="B122" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="123" spans="2:2">
       <c r="B123" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="124" spans="2:2">
       <c r="B124" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="125" spans="2:2">
       <c r="B125" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="126" spans="2:2">
       <c r="B126" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="127" spans="2:2">
       <c r="B127" t="s">
-        <v>743</v>
+        <v>234</v>
       </c>
     </row>
     <row r="128" spans="2:2">
       <c r="B128" t="s">
-        <v>236</v>
+        <v>746</v>
       </c>
     </row>
     <row r="129" spans="2:2">
       <c r="B129" t="s">
-        <v>733</v>
+        <v>236</v>
       </c>
     </row>
     <row r="130" spans="2:2">
       <c r="B130" t="s">
-        <v>238</v>
+        <v>736</v>
       </c>
     </row>
     <row r="131" spans="2:2">
       <c r="B131" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="132" spans="2:2">
       <c r="B132" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="133" spans="2:2">
       <c r="B133" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="134" spans="2:2">
       <c r="B134" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="135" spans="2:2">
       <c r="B135" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="136" spans="2:2">
       <c r="B136" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="137" spans="2:2">
       <c r="B137" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="138" spans="2:2">
       <c r="B138" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="139" spans="2:2">
       <c r="B139" t="s">
-        <v>628</v>
+        <v>255</v>
       </c>
     </row>
     <row r="140" spans="2:2">
       <c r="B140" t="s">
-        <v>257</v>
+        <v>628</v>
       </c>
     </row>
     <row r="141" spans="2:2">
       <c r="B141" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="142" spans="2:2">
       <c r="B142" t="s">
-        <v>630</v>
+        <v>259</v>
       </c>
     </row>
     <row r="143" spans="2:2">
       <c r="B143" t="s">
-        <v>261</v>
+        <v>630</v>
       </c>
     </row>
     <row r="144" spans="2:2">
       <c r="B144" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="145" spans="2:2">
       <c r="B145" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="146" spans="2:2">
       <c r="B146" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="147" spans="2:2">
       <c r="B147" t="s">
-        <v>633</v>
+        <v>269</v>
       </c>
     </row>
     <row r="148" spans="2:2">
       <c r="B148" t="s">
-        <v>271</v>
+        <v>633</v>
       </c>
     </row>
     <row r="149" spans="2:2">
       <c r="B149" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="150" spans="2:2">
       <c r="B150" t="s">
-        <v>735</v>
+        <v>273</v>
       </c>
     </row>
     <row r="151" spans="2:2">
       <c r="B151" t="s">
-        <v>275</v>
+        <v>738</v>
       </c>
     </row>
     <row r="152" spans="2:2">
       <c r="B152" t="s">
-        <v>699</v>
+        <v>275</v>
       </c>
     </row>
     <row r="153" spans="2:2">
       <c r="B153" t="s">
-        <v>277</v>
+        <v>702</v>
       </c>
     </row>
     <row r="154" spans="2:2">
       <c r="B154" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="155" spans="2:2">
       <c r="B155" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="156" spans="2:2">
       <c r="B156" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="157" spans="2:2">
       <c r="B157" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="158" spans="2:2">
       <c r="B158" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="159" spans="2:2">
       <c r="B159" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="160" spans="2:2">
       <c r="B160" t="s">
-        <v>636</v>
+        <v>290</v>
       </c>
     </row>
     <row r="161" spans="2:2">
       <c r="B161" t="s">
-        <v>292</v>
+        <v>636</v>
       </c>
     </row>
     <row r="162" spans="2:2">
       <c r="B162" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="163" spans="2:2">
       <c r="B163" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="164" spans="2:2">
       <c r="B164" t="s">
-        <v>638</v>
+        <v>296</v>
       </c>
     </row>
     <row r="165" spans="2:2">
       <c r="B165" t="s">
-        <v>298</v>
+        <v>638</v>
       </c>
     </row>
     <row r="166" spans="2:2">
       <c r="B166" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="167" spans="2:2">
       <c r="B167" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="168" spans="2:2">
       <c r="B168" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="169" spans="2:2">
       <c r="B169" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="170" spans="2:2">
       <c r="B170" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="171" spans="2:2">
       <c r="B171" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="172" spans="2:2">
       <c r="B172" t="s">
-        <v>641</v>
+        <v>310</v>
       </c>
     </row>
     <row r="173" spans="2:2">
       <c r="B173" t="s">
-        <v>312</v>
+        <v>641</v>
       </c>
     </row>
     <row r="174" spans="2:2">
       <c r="B174" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="175" spans="2:2">
       <c r="B175" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="176" spans="2:2">
       <c r="B176" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="177" spans="2:2">
       <c r="B177" t="s">
-        <v>746</v>
+        <v>318</v>
       </c>
     </row>
     <row r="178" spans="2:2">
       <c r="B178" t="s">
-        <v>320</v>
+        <v>749</v>
       </c>
     </row>
     <row r="179" spans="2:2">
       <c r="B179" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="180" spans="2:2">
       <c r="B180" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="181" spans="2:2">
       <c r="B181" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="182" spans="2:2">
       <c r="B182" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="183" spans="2:2">
       <c r="B183" t="s">
-        <v>644</v>
+        <v>328</v>
       </c>
     </row>
     <row r="184" spans="2:2">
       <c r="B184" t="s">
-        <v>330</v>
+        <v>644</v>
       </c>
     </row>
     <row r="185" spans="2:2">
       <c r="B185" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="186" spans="2:2">
       <c r="B186" t="s">
-        <v>646</v>
+        <v>332</v>
       </c>
     </row>
     <row r="187" spans="2:2">
       <c r="B187" t="s">
-        <v>333</v>
+        <v>646</v>
       </c>
     </row>
     <row r="188" spans="2:2">
       <c r="B188" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="189" spans="2:2">
       <c r="B189" t="s">
-        <v>702</v>
+        <v>335</v>
       </c>
     </row>
     <row r="190" spans="2:2">
       <c r="B190" t="s">
-        <v>649</v>
+        <v>705</v>
       </c>
     </row>
     <row r="191" spans="2:2">
       <c r="B191" t="s">
-        <v>337</v>
+        <v>649</v>
       </c>
     </row>
     <row r="192" spans="2:2">
       <c r="B192" t="s">
-        <v>652</v>
+        <v>337</v>
       </c>
     </row>
     <row r="193" spans="2:2">
       <c r="B193" t="s">
-        <v>338</v>
+        <v>652</v>
       </c>
     </row>
     <row r="194" spans="2:2">
       <c r="B194" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="195" spans="2:2">
       <c r="B195" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="196" spans="2:2">
       <c r="B196" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="197" spans="2:2">
       <c r="B197" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="198" spans="2:2">
       <c r="B198" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="199" spans="2:2">
       <c r="B199" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="200" spans="2:2">
       <c r="B200" t="s">
-        <v>705</v>
+        <v>351</v>
       </c>
     </row>
     <row r="201" spans="2:2">
       <c r="B201" t="s">
-        <v>353</v>
+        <v>708</v>
       </c>
     </row>
     <row r="202" spans="2:2">
       <c r="B202" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="203" spans="2:2">
       <c r="B203" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="204" spans="2:2">
       <c r="B204" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="205" spans="2:2">
       <c r="B205" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="206" spans="2:2">
       <c r="B206" t="s">
-        <v>654</v>
+        <v>361</v>
       </c>
     </row>
     <row r="207" spans="2:2">
       <c r="B207" t="s">
-        <v>363</v>
+        <v>654</v>
       </c>
     </row>
     <row r="208" spans="2:2">
       <c r="B208" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="209" spans="2:2">
       <c r="B209" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="210" spans="2:2">
       <c r="B210" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="211" spans="2:2">
       <c r="B211" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="212" spans="2:2">
       <c r="B212" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="213" spans="2:2">
       <c r="B213" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="214" spans="2:2">
       <c r="B214" t="s">
-        <v>657</v>
+        <v>374</v>
       </c>
     </row>
     <row r="215" spans="2:2">
       <c r="B215" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
     <row r="216" spans="2:2">
       <c r="B216" t="s">
-        <v>377</v>
+        <v>660</v>
       </c>
     </row>
     <row r="217" spans="2:2">
       <c r="B217" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="218" spans="2:2">
       <c r="B218" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="219" spans="2:2">
       <c r="B219" t="s">
-        <v>737</v>
+        <v>380</v>
       </c>
     </row>
     <row r="220" spans="2:2">
       <c r="B220" t="s">
-        <v>382</v>
+        <v>740</v>
       </c>
     </row>
     <row r="221" spans="2:2">
       <c r="B221" t="s">
-        <v>750</v>
+        <v>382</v>
       </c>
     </row>
     <row r="222" spans="2:2">
       <c r="B222" t="s">
-        <v>384</v>
+        <v>753</v>
       </c>
     </row>
     <row r="223" spans="2:2">
       <c r="B223" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="224" spans="2:2">
       <c r="B224" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="225" spans="2:2">
       <c r="B225" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="226" spans="2:2">
       <c r="B226" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="227" spans="2:2">
       <c r="B227" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="228" spans="2:2">
       <c r="B228" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="229" spans="2:2">
       <c r="B229" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="230" spans="2:2">
       <c r="B230" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="231" spans="2:2">
       <c r="B231" t="s">
-        <v>663</v>
+        <v>400</v>
       </c>
     </row>
     <row r="232" spans="2:2">
       <c r="B232" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
     </row>
     <row r="233" spans="2:2">
       <c r="B233" t="s">
-        <v>402</v>
+        <v>666</v>
       </c>
     </row>
     <row r="234" spans="2:2">
       <c r="B234" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="235" spans="2:2">
       <c r="B235" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="236" spans="2:2">
       <c r="B236" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="237" spans="2:2">
       <c r="B237" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="238" spans="2:2">
       <c r="B238" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="239" spans="2:2">
       <c r="B239" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="240" spans="2:2">
       <c r="B240" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="241" spans="2:2">
       <c r="B241" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="242" spans="2:2">
       <c r="B242" t="s">
-        <v>707</v>
+        <v>420</v>
       </c>
     </row>
     <row r="243" spans="2:2">
       <c r="B243" t="s">
-        <v>669</v>
+        <v>710</v>
       </c>
     </row>
     <row r="244" spans="2:2">
       <c r="B244" t="s">
-        <v>421</v>
+        <v>669</v>
       </c>
     </row>
     <row r="245" spans="2:2">
       <c r="B245" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="246" spans="2:2">
       <c r="B246" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="247" spans="2:2">
       <c r="B247" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="248" spans="2:2">
       <c r="B248" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="249" spans="2:2">
       <c r="B249" t="s">
-        <v>671</v>
+        <v>429</v>
       </c>
     </row>
     <row r="250" spans="2:2">
       <c r="B250" t="s">
-        <v>431</v>
+        <v>671</v>
       </c>
     </row>
     <row r="251" spans="2:2">
       <c r="B251" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="252" spans="2:2">
       <c r="B252" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="253" spans="2:2">
       <c r="B253" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="254" spans="2:2">
       <c r="B254" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="255" spans="2:2">
       <c r="B255" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="256" spans="2:2">
       <c r="B256" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="257" spans="2:2">
       <c r="B257" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="258" spans="2:2">
       <c r="B258" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="259" spans="2:2">
       <c r="B259" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="260" spans="2:2">
       <c r="B260" t="s">
-        <v>673</v>
+        <v>450</v>
       </c>
     </row>
     <row r="261" spans="2:2">
       <c r="B261" t="s">
-        <v>452</v>
+        <v>673</v>
       </c>
     </row>
     <row r="262" spans="2:2">
       <c r="B262" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="263" spans="2:2">
       <c r="B263" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="264" spans="2:2">
       <c r="B264" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="265" spans="2:2">
       <c r="B265" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="266" spans="2:2">
       <c r="B266" t="s">
-        <v>676</v>
+        <v>460</v>
       </c>
     </row>
     <row r="267" spans="2:2">
       <c r="B267" t="s">
-        <v>462</v>
+        <v>676</v>
       </c>
     </row>
     <row r="268" spans="2:2">
       <c r="B268" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="269" spans="2:2">
       <c r="B269" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="270" spans="2:2">
       <c r="B270" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="271" spans="2:2">
       <c r="B271" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="272" spans="2:2">
       <c r="B272" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="273" spans="2:2">
       <c r="B273" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="274" spans="2:2">
       <c r="B274" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="275" spans="2:2">
       <c r="B275" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="276" spans="2:2">
       <c r="B276" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="277" spans="2:2">
       <c r="B277" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="278" spans="2:2">
       <c r="B278" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="279" spans="2:2">
       <c r="B279" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="280" spans="2:2">
       <c r="B280" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="281" spans="2:2">
       <c r="B281" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="282" spans="2:2">
       <c r="B282" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="283" spans="2:2">
       <c r="B283" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="284" spans="2:2">
       <c r="B284" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="285" spans="2:2">
       <c r="B285" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="286" spans="2:2">
       <c r="B286" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="287" spans="2:2">
       <c r="B287" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="288" spans="2:2">
       <c r="B288" t="s">
-        <v>754</v>
+        <v>503</v>
       </c>
     </row>
     <row r="289" spans="2:2">
       <c r="B289" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="290" spans="2:2">
       <c r="B290" t="s">
-        <v>505</v>
+        <v>761</v>
       </c>
     </row>
     <row r="291" spans="2:2">
       <c r="B291" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="292" spans="2:2">
       <c r="B292" t="s">
-        <v>760</v>
+        <v>507</v>
       </c>
     </row>
     <row r="293" spans="2:2">
       <c r="B293" t="s">
-        <v>679</v>
+        <v>763</v>
       </c>
     </row>
     <row r="294" spans="2:2">
       <c r="B294" t="s">
-        <v>509</v>
+        <v>679</v>
       </c>
     </row>
     <row r="295" spans="2:2">
       <c r="B295" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
     <row r="296" spans="2:2">
       <c r="B296" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="297" spans="2:2">
       <c r="B297" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="298" spans="2:2">
       <c r="B298" t="s">
-        <v>709</v>
+        <v>515</v>
       </c>
     </row>
     <row r="299" spans="2:2">
       <c r="B299" t="s">
-        <v>517</v>
+        <v>712</v>
       </c>
     </row>
     <row r="300" spans="2:2">
       <c r="B300" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="301" spans="2:2">
       <c r="B301" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="302" spans="2:2">
       <c r="B302" t="s">
-        <v>711</v>
+        <v>521</v>
       </c>
     </row>
     <row r="303" spans="2:2">
       <c r="B303" t="s">
-        <v>523</v>
+        <v>714</v>
       </c>
     </row>
     <row r="304" spans="2:2">
       <c r="B304" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="305" spans="2:2">
       <c r="B305" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="306" spans="2:2">
       <c r="B306" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="307" spans="2:2">
       <c r="B307" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="308" spans="2:2">
       <c r="B308" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="309" spans="2:2">
       <c r="B309" t="s">
-        <v>713</v>
+        <v>533</v>
       </c>
     </row>
     <row r="310" spans="2:2">
       <c r="B310" t="s">
-        <v>535</v>
+        <v>716</v>
       </c>
     </row>
     <row r="311" spans="2:2">
       <c r="B311" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="312" spans="2:2">
       <c r="B312" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="313" spans="2:2">
       <c r="B313" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="314" spans="2:2">
       <c r="B314" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="315" spans="2:2">
       <c r="B315" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
     <row r="316" spans="2:2">
       <c r="B316" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
     </row>
     <row r="317" spans="2:2">
       <c r="B317" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="318" spans="2:2">
       <c r="B318" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="319" spans="2:2">
       <c r="B319" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="320" spans="2:2">
       <c r="B320" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
     </row>
     <row r="321" spans="2:2">
       <c r="B321" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="322" spans="2:2">
       <c r="B322" t="s">
-        <v>682</v>
+        <v>557</v>
       </c>
     </row>
     <row r="323" spans="2:2">
       <c r="B323" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="324" spans="2:2">
       <c r="B324" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
     </row>
     <row r="325" spans="2:2">
       <c r="B325" t="s">
-        <v>559</v>
+        <v>687</v>
       </c>
     </row>
     <row r="326" spans="2:2">
       <c r="B326" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
     <row r="327" spans="2:2">
       <c r="B327" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="328" spans="2:2">
       <c r="B328" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="329" spans="2:2">
       <c r="B329" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="330" spans="2:2">
       <c r="B330" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="331" spans="2:2">
       <c r="B331" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="332" spans="2:2">
       <c r="B332" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="333" spans="2:2">
       <c r="B333" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="334" spans="2:2">
       <c r="B334" t="s">
-        <v>740</v>
+        <v>575</v>
       </c>
     </row>
     <row r="335" spans="2:2">
       <c r="B335" t="s">
-        <v>577</v>
+        <v>743</v>
       </c>
     </row>
     <row r="336" spans="2:2">
       <c r="B336" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
     </row>
     <row r="337" spans="1:2">
       <c r="B337" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="338" spans="1:2">
       <c r="B338" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="339" spans="1:2">
       <c r="B339" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
     </row>
     <row r="340" spans="1:2">
       <c r="B340" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
     </row>
     <row r="341" spans="1:2">
       <c r="B341" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="342" spans="1:2">
       <c r="B342" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="343" spans="1:2">
       <c r="B343" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="344" spans="1:2">
       <c r="B344" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
     </row>
     <row r="345" spans="1:2">
       <c r="B345" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="346" spans="1:2">
+      <c r="B346" t="s">
         <v>598</v>
       </c>
     </row>
-    <row r="347" spans="1:2">
-      <c r="A347" t="s">
-        <v>766</v>
-      </c>
-      <c r="B347" t="s">
+    <row r="348" spans="1:2">
+      <c r="A348" t="s">
+        <v>769</v>
+      </c>
+      <c r="B348" t="s">
         <v>696</v>
       </c>
     </row>
-    <row r="349" spans="1:2">
-      <c r="A349" t="s">
-        <v>767</v>
-      </c>
-      <c r="B349" t="s">
+    <row r="350" spans="1:2">
+      <c r="A350" t="s">
+        <v>770</v>
+      </c>
+      <c r="B350" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="350" spans="1:2">
-      <c r="B350" t="s">
+    <row r="351" spans="1:2">
+      <c r="B351" t="s">
         <v>676</v>
       </c>
     </row>
-    <row r="352" spans="1:2">
-      <c r="A352" t="s">
-        <v>768</v>
-      </c>
-      <c r="B352" t="s">
+    <row r="353" spans="1:2">
+      <c r="A353" t="s">
+        <v>771</v>
+      </c>
+      <c r="B353" t="s">
         <v>619</v>
       </c>
     </row>
-    <row r="353" spans="2:2">
-      <c r="B353" t="s">
-        <v>733</v>
-      </c>
-    </row>
-    <row r="354" spans="2:2">
+    <row r="354" spans="1:2">
       <c r="B354" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="355" spans="1:2">
+      <c r="B355" t="s">
         <v>633</v>
       </c>
     </row>
-    <row r="355" spans="2:2">
-      <c r="B355" t="s">
+    <row r="356" spans="1:2">
+      <c r="B356" t="s">
         <v>644</v>
       </c>
     </row>
@@ -10111,7 +10125,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="110.7109375" customWidth="1"/>
@@ -10197,7 +10211,7 @@
         <v>699</v>
       </c>
       <c r="B6">
-        <v>1.88</v>
+        <v>1.75</v>
       </c>
       <c r="C6" t="s">
         <v>700</v>
@@ -10214,7 +10228,7 @@
         <v>702</v>
       </c>
       <c r="B7">
-        <v>2.66</v>
+        <v>1.88</v>
       </c>
       <c r="C7" t="s">
         <v>703</v>
@@ -10231,7 +10245,7 @@
         <v>705</v>
       </c>
       <c r="B8">
-        <v>1.76</v>
+        <v>2.66</v>
       </c>
       <c r="C8" t="s">
         <v>706</v>
@@ -10240,75 +10254,92 @@
         <v>8</v>
       </c>
       <c r="E8" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="B9">
-        <v>1.84</v>
+        <v>1.76</v>
       </c>
       <c r="C9" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="D9" t="s">
         <v>8</v>
       </c>
       <c r="E9" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="B10">
-        <v>2</v>
+        <v>1.84</v>
       </c>
       <c r="C10" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="D10" t="s">
         <v>8</v>
       </c>
       <c r="E10" t="s">
-        <v>643</v>
+        <v>704</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B11">
-        <v>1.92</v>
+        <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="D11" t="s">
         <v>8</v>
       </c>
       <c r="E11" t="s">
-        <v>701</v>
+        <v>643</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="B12">
+        <v>1.92</v>
+      </c>
+      <c r="C12" t="s">
+        <v>715</v>
+      </c>
+      <c r="D12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>716</v>
+      </c>
+      <c r="B13">
         <v>1.77</v>
       </c>
-      <c r="C12" t="s">
-        <v>714</v>
-      </c>
-      <c r="D12" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" t="s">
-        <v>701</v>
+      <c r="C13" t="s">
+        <v>717</v>
+      </c>
+      <c r="D13" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" t="s">
+        <v>704</v>
       </c>
     </row>
   </sheetData>
@@ -10328,7 +10359,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10350,19 +10381,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="B3">
         <v>2.2</v>
       </c>
       <c r="C3" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
     </row>
   </sheetData>
@@ -10382,7 +10413,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10404,19 +10435,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="B3">
         <v>1.32</v>
       </c>
       <c r="C3" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
     </row>
   </sheetData>
@@ -10436,7 +10467,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10458,19 +10489,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="B3">
         <v>2.45</v>
       </c>
       <c r="C3" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
     </row>
   </sheetData>
@@ -10490,7 +10521,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10512,47 +10543,47 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="B3">
         <v>1.9</v>
       </c>
       <c r="C3" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
       <c r="B4">
         <v>2.11</v>
       </c>
       <c r="C4" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="B5">
         <v>2.7</v>
       </c>
       <c r="C5" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -10563,13 +10594,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="B6">
         <v>2.58</v>
       </c>
       <c r="C6" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -10580,30 +10611,30 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="B7">
         <v>1.93</v>
       </c>
       <c r="C7" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="B8">
         <v>2.05</v>
       </c>
       <c r="C8" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
@@ -10629,7 +10660,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10651,13 +10682,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="B3">
         <v>0.93</v>
       </c>
       <c r="C3" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -10683,7 +10714,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10705,19 +10736,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="B3">
         <v>2.17</v>
       </c>
       <c r="C3" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
weekly update, 2022-05-11, SARS-CoV-2
</commit_message>
<xml_diff>
--- a/pdb/nsp3/SARS-CoV-2/domains_and_infos_of_nsp3.xlsx
+++ b/pdb/nsp3/SARS-CoV-2/domains_and_infos_of_nsp3.xlsx
@@ -13,20 +13,21 @@
     <sheet name="nsp3_betaSM-M_" sheetId="4" r:id="rId4"/>
     <sheet name="nsp3_DPUP_nsp3_Ubl2_" sheetId="5" r:id="rId5"/>
     <sheet name="nsp3_NAB_" sheetId="6" r:id="rId6"/>
-    <sheet name="nsp3_PL2pro_" sheetId="7" r:id="rId7"/>
-    <sheet name="nsp3_Macro1_nsp3_PL2pro_" sheetId="8" r:id="rId8"/>
-    <sheet name="nsp3_Y3_" sheetId="9" r:id="rId9"/>
-    <sheet name="None" sheetId="10" r:id="rId10"/>
-    <sheet name="nsp3_PL2pro_nsp3_Ubl2_" sheetId="11" r:id="rId11"/>
-    <sheet name="nsp3_Ubl1_" sheetId="12" r:id="rId12"/>
-    <sheet name="Organisms" sheetId="13" r:id="rId13"/>
+    <sheet name="multi-domain1" sheetId="7" r:id="rId7"/>
+    <sheet name="nsp3_PL2pro_" sheetId="8" r:id="rId8"/>
+    <sheet name="nsp3_Macro1_nsp3_PL2pro_" sheetId="9" r:id="rId9"/>
+    <sheet name="nsp3_Y3_" sheetId="10" r:id="rId10"/>
+    <sheet name="None" sheetId="11" r:id="rId11"/>
+    <sheet name="nsp3_PL2pro_nsp3_Ubl2_" sheetId="12" r:id="rId12"/>
+    <sheet name="nsp3_Ubl1_" sheetId="13" r:id="rId13"/>
+    <sheet name="Organisms" sheetId="14" r:id="rId14"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1806" uniqueCount="772">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1819" uniqueCount="776">
   <si>
     <t>nsp3_Macro1_</t>
   </si>
@@ -2218,6 +2219,18 @@
     <t>2021-01-20</t>
   </si>
   <si>
+    <t>nsp3_PL2pro_nsp3_HVR_nsp3_Macro1_nsp3_Macro2_nsp3_Macro3_nsp3_Ubl2_nsp3_betaSM-C_nsp3_pred_Ecto_nsp3_Y1-CoV-Y-N_nsp3_Y3_</t>
+  </si>
+  <si>
+    <t>7uv5</t>
+  </si>
+  <si>
+    <t>THE CRYSTAL STRUCTURE OF PAPAIN-LIKE PROTEASE OF SARS COV-2, C111S/D286N MUTANT, IN COMPLEX WITH A LYS48-LINKED DI-UBIQUITIN</t>
+  </si>
+  <si>
+    <t>2022-04-29</t>
+  </si>
+  <si>
     <t>nsp3_PL2pro_</t>
   </si>
   <si>
@@ -2335,13 +2348,13 @@
     <t xml:space="preserve">severe acute respiratory syndrome coronavirus2 </t>
   </si>
   <si>
+    <t>homo sapiens</t>
+  </si>
+  <si>
     <t>mus musculus</t>
   </si>
   <si>
     <t>synthetic construct</t>
-  </si>
-  <si>
-    <t>homo sapiens</t>
   </si>
 </sst>
 </file>
@@ -7607,7 +7620,7 @@
         <v>753</v>
       </c>
       <c r="B3">
-        <v>2.72</v>
+        <v>2.17</v>
       </c>
       <c r="C3" t="s">
         <v>754</v>
@@ -7661,7 +7674,7 @@
         <v>757</v>
       </c>
       <c r="B3">
-        <v>2.68</v>
+        <v>2.72</v>
       </c>
       <c r="C3" t="s">
         <v>758</v>
@@ -7679,6 +7692,60 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="110.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>761</v>
+      </c>
+      <c r="B3">
+        <v>2.68</v>
+      </c>
+      <c r="C3" t="s">
+        <v>762</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>763</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -7690,7 +7757,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -7712,13 +7779,13 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="B3">
         <v>3.21</v>
       </c>
       <c r="C3" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
@@ -7729,19 +7796,19 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B4">
         <v>2.73</v>
       </c>
       <c r="C4" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
     </row>
   </sheetData>
@@ -7749,9 +7816,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B356"/>
+  <dimension ref="A1:B359"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.7109375" customWidth="1"/>
@@ -7759,12 +7826,12 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
@@ -7772,7 +7839,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>768</v>
+        <v>772</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
@@ -8005,1207 +8072,1207 @@
     </row>
     <row r="49" spans="2:2">
       <c r="B49" t="s">
-        <v>90</v>
+        <v>731</v>
       </c>
     </row>
     <row r="50" spans="2:2">
       <c r="B50" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="51" spans="2:2">
       <c r="B51" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="52" spans="2:2">
       <c r="B52" t="s">
-        <v>696</v>
+        <v>94</v>
       </c>
     </row>
     <row r="53" spans="2:2">
       <c r="B53" t="s">
-        <v>96</v>
+        <v>696</v>
       </c>
     </row>
     <row r="54" spans="2:2">
       <c r="B54" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="2:2">
       <c r="B55" t="s">
-        <v>731</v>
+        <v>98</v>
       </c>
     </row>
     <row r="56" spans="2:2">
       <c r="B56" t="s">
-        <v>100</v>
+        <v>735</v>
       </c>
     </row>
     <row r="57" spans="2:2">
       <c r="B57" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58" spans="2:2">
       <c r="B58" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="2:2">
       <c r="B59" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="60" spans="2:2">
       <c r="B60" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="61" spans="2:2">
       <c r="B61" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="62" spans="2:2">
       <c r="B62" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="63" spans="2:2">
       <c r="B63" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="64" spans="2:2">
       <c r="B64" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="65" spans="2:2">
       <c r="B65" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="66" spans="2:2">
       <c r="B66" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="67" spans="2:2">
       <c r="B67" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="68" spans="2:2">
       <c r="B68" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="69" spans="2:2">
       <c r="B69" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="70" spans="2:2">
       <c r="B70" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="71" spans="2:2">
       <c r="B71" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="72" spans="2:2">
       <c r="B72" t="s">
-        <v>613</v>
+        <v>131</v>
       </c>
     </row>
     <row r="73" spans="2:2">
       <c r="B73" t="s">
-        <v>134</v>
+        <v>613</v>
       </c>
     </row>
     <row r="74" spans="2:2">
       <c r="B74" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="75" spans="2:2">
       <c r="B75" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="76" spans="2:2">
       <c r="B76" t="s">
-        <v>616</v>
+        <v>138</v>
       </c>
     </row>
     <row r="77" spans="2:2">
       <c r="B77" t="s">
-        <v>140</v>
+        <v>616</v>
       </c>
     </row>
     <row r="78" spans="2:2">
       <c r="B78" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="79" spans="2:2">
       <c r="B79" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="80" spans="2:2">
       <c r="B80" t="s">
-        <v>619</v>
+        <v>144</v>
       </c>
     </row>
     <row r="81" spans="2:2">
       <c r="B81" t="s">
-        <v>146</v>
+        <v>619</v>
       </c>
     </row>
     <row r="82" spans="2:2">
       <c r="B82" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="83" spans="2:2">
       <c r="B83" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="84" spans="2:2">
       <c r="B84" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="85" spans="2:2">
       <c r="B85" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="86" spans="2:2">
       <c r="B86" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="87" spans="2:2">
       <c r="B87" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="88" spans="2:2">
       <c r="B88" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="89" spans="2:2">
       <c r="B89" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="90" spans="2:2">
       <c r="B90" t="s">
-        <v>622</v>
+        <v>163</v>
       </c>
     </row>
     <row r="91" spans="2:2">
       <c r="B91" t="s">
-        <v>165</v>
+        <v>622</v>
       </c>
     </row>
     <row r="92" spans="2:2">
       <c r="B92" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="93" spans="2:2">
       <c r="B93" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="94" spans="2:2">
       <c r="B94" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="95" spans="2:2">
       <c r="B95" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="96" spans="2:2">
       <c r="B96" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="97" spans="2:2">
       <c r="B97" t="s">
-        <v>625</v>
+        <v>175</v>
       </c>
     </row>
     <row r="98" spans="2:2">
       <c r="B98" t="s">
-        <v>699</v>
+        <v>625</v>
       </c>
     </row>
     <row r="99" spans="2:2">
       <c r="B99" t="s">
-        <v>177</v>
+        <v>699</v>
       </c>
     </row>
     <row r="100" spans="2:2">
       <c r="B100" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="101" spans="2:2">
       <c r="B101" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="102" spans="2:2">
       <c r="B102" t="s">
-        <v>734</v>
+        <v>181</v>
       </c>
     </row>
     <row r="103" spans="2:2">
       <c r="B103" t="s">
-        <v>183</v>
+        <v>738</v>
       </c>
     </row>
     <row r="104" spans="2:2">
       <c r="B104" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="105" spans="2:2">
       <c r="B105" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="106" spans="2:2">
       <c r="B106" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="107" spans="2:2">
       <c r="B107" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="108" spans="2:2">
       <c r="B108" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="109" spans="2:2">
       <c r="B109" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="110" spans="2:2">
       <c r="B110" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="111" spans="2:2">
       <c r="B111" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
     </row>
     <row r="112" spans="2:2">
       <c r="B112" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="113" spans="2:2">
       <c r="B113" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="114" spans="2:2">
       <c r="B114" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="115" spans="2:2">
       <c r="B115" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="116" spans="2:2">
       <c r="B116" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="117" spans="2:2">
       <c r="B117" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="118" spans="2:2">
       <c r="B118" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="119" spans="2:2">
       <c r="B119" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="120" spans="2:2">
       <c r="B120" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="121" spans="2:2">
       <c r="B121" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="122" spans="2:2">
       <c r="B122" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="123" spans="2:2">
       <c r="B123" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="124" spans="2:2">
       <c r="B124" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="125" spans="2:2">
       <c r="B125" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="126" spans="2:2">
       <c r="B126" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="127" spans="2:2">
       <c r="B127" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="128" spans="2:2">
       <c r="B128" t="s">
-        <v>746</v>
+        <v>234</v>
       </c>
     </row>
     <row r="129" spans="2:2">
       <c r="B129" t="s">
-        <v>236</v>
+        <v>750</v>
       </c>
     </row>
     <row r="130" spans="2:2">
       <c r="B130" t="s">
-        <v>736</v>
+        <v>236</v>
       </c>
     </row>
     <row r="131" spans="2:2">
       <c r="B131" t="s">
-        <v>238</v>
+        <v>740</v>
       </c>
     </row>
     <row r="132" spans="2:2">
       <c r="B132" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="133" spans="2:2">
       <c r="B133" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="134" spans="2:2">
       <c r="B134" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="135" spans="2:2">
       <c r="B135" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="136" spans="2:2">
       <c r="B136" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="137" spans="2:2">
       <c r="B137" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="138" spans="2:2">
       <c r="B138" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="139" spans="2:2">
       <c r="B139" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="140" spans="2:2">
       <c r="B140" t="s">
-        <v>628</v>
+        <v>255</v>
       </c>
     </row>
     <row r="141" spans="2:2">
       <c r="B141" t="s">
-        <v>257</v>
+        <v>628</v>
       </c>
     </row>
     <row r="142" spans="2:2">
       <c r="B142" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="143" spans="2:2">
       <c r="B143" t="s">
-        <v>630</v>
+        <v>259</v>
       </c>
     </row>
     <row r="144" spans="2:2">
       <c r="B144" t="s">
-        <v>261</v>
+        <v>630</v>
       </c>
     </row>
     <row r="145" spans="2:2">
       <c r="B145" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="146" spans="2:2">
       <c r="B146" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="147" spans="2:2">
       <c r="B147" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="148" spans="2:2">
       <c r="B148" t="s">
-        <v>633</v>
+        <v>269</v>
       </c>
     </row>
     <row r="149" spans="2:2">
       <c r="B149" t="s">
-        <v>271</v>
+        <v>633</v>
       </c>
     </row>
     <row r="150" spans="2:2">
       <c r="B150" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="151" spans="2:2">
       <c r="B151" t="s">
-        <v>738</v>
+        <v>273</v>
       </c>
     </row>
     <row r="152" spans="2:2">
       <c r="B152" t="s">
-        <v>275</v>
+        <v>742</v>
       </c>
     </row>
     <row r="153" spans="2:2">
       <c r="B153" t="s">
-        <v>702</v>
+        <v>275</v>
       </c>
     </row>
     <row r="154" spans="2:2">
       <c r="B154" t="s">
-        <v>277</v>
+        <v>702</v>
       </c>
     </row>
     <row r="155" spans="2:2">
       <c r="B155" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="156" spans="2:2">
       <c r="B156" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="157" spans="2:2">
       <c r="B157" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="158" spans="2:2">
       <c r="B158" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="159" spans="2:2">
       <c r="B159" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="160" spans="2:2">
       <c r="B160" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
     </row>
     <row r="161" spans="2:2">
       <c r="B161" t="s">
-        <v>636</v>
+        <v>290</v>
       </c>
     </row>
     <row r="162" spans="2:2">
       <c r="B162" t="s">
-        <v>292</v>
+        <v>636</v>
       </c>
     </row>
     <row r="163" spans="2:2">
       <c r="B163" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="164" spans="2:2">
       <c r="B164" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="165" spans="2:2">
       <c r="B165" t="s">
-        <v>638</v>
+        <v>296</v>
       </c>
     </row>
     <row r="166" spans="2:2">
       <c r="B166" t="s">
-        <v>298</v>
+        <v>638</v>
       </c>
     </row>
     <row r="167" spans="2:2">
       <c r="B167" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
     </row>
     <row r="168" spans="2:2">
       <c r="B168" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
     </row>
     <row r="169" spans="2:2">
       <c r="B169" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="170" spans="2:2">
       <c r="B170" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
     </row>
     <row r="171" spans="2:2">
       <c r="B171" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
     </row>
     <row r="172" spans="2:2">
       <c r="B172" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="173" spans="2:2">
       <c r="B173" t="s">
-        <v>641</v>
+        <v>310</v>
       </c>
     </row>
     <row r="174" spans="2:2">
       <c r="B174" t="s">
-        <v>312</v>
+        <v>641</v>
       </c>
     </row>
     <row r="175" spans="2:2">
       <c r="B175" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="176" spans="2:2">
       <c r="B176" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
     </row>
     <row r="177" spans="2:2">
       <c r="B177" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
     </row>
     <row r="178" spans="2:2">
       <c r="B178" t="s">
-        <v>749</v>
+        <v>318</v>
       </c>
     </row>
     <row r="179" spans="2:2">
       <c r="B179" t="s">
-        <v>320</v>
+        <v>753</v>
       </c>
     </row>
     <row r="180" spans="2:2">
       <c r="B180" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
     </row>
     <row r="181" spans="2:2">
       <c r="B181" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
     </row>
     <row r="182" spans="2:2">
       <c r="B182" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
     </row>
     <row r="183" spans="2:2">
       <c r="B183" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
     </row>
     <row r="184" spans="2:2">
       <c r="B184" t="s">
-        <v>644</v>
+        <v>328</v>
       </c>
     </row>
     <row r="185" spans="2:2">
       <c r="B185" t="s">
-        <v>330</v>
+        <v>644</v>
       </c>
     </row>
     <row r="186" spans="2:2">
       <c r="B186" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
     </row>
     <row r="187" spans="2:2">
       <c r="B187" t="s">
-        <v>646</v>
+        <v>332</v>
       </c>
     </row>
     <row r="188" spans="2:2">
       <c r="B188" t="s">
-        <v>333</v>
+        <v>646</v>
       </c>
     </row>
     <row r="189" spans="2:2">
       <c r="B189" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
     </row>
     <row r="190" spans="2:2">
       <c r="B190" t="s">
-        <v>705</v>
+        <v>335</v>
       </c>
     </row>
     <row r="191" spans="2:2">
       <c r="B191" t="s">
-        <v>649</v>
+        <v>705</v>
       </c>
     </row>
     <row r="192" spans="2:2">
       <c r="B192" t="s">
-        <v>337</v>
+        <v>649</v>
       </c>
     </row>
     <row r="193" spans="2:2">
       <c r="B193" t="s">
-        <v>652</v>
+        <v>337</v>
       </c>
     </row>
     <row r="194" spans="2:2">
       <c r="B194" t="s">
-        <v>338</v>
+        <v>652</v>
       </c>
     </row>
     <row r="195" spans="2:2">
       <c r="B195" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="196" spans="2:2">
       <c r="B196" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
     </row>
     <row r="197" spans="2:2">
       <c r="B197" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="198" spans="2:2">
       <c r="B198" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="199" spans="2:2">
       <c r="B199" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="200" spans="2:2">
       <c r="B200" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="201" spans="2:2">
       <c r="B201" t="s">
-        <v>708</v>
+        <v>351</v>
       </c>
     </row>
     <row r="202" spans="2:2">
       <c r="B202" t="s">
-        <v>353</v>
+        <v>708</v>
       </c>
     </row>
     <row r="203" spans="2:2">
       <c r="B203" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
     </row>
     <row r="204" spans="2:2">
       <c r="B204" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="205" spans="2:2">
       <c r="B205" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="206" spans="2:2">
       <c r="B206" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
     </row>
     <row r="207" spans="2:2">
       <c r="B207" t="s">
-        <v>654</v>
+        <v>361</v>
       </c>
     </row>
     <row r="208" spans="2:2">
       <c r="B208" t="s">
-        <v>363</v>
+        <v>654</v>
       </c>
     </row>
     <row r="209" spans="2:2">
       <c r="B209" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="210" spans="2:2">
       <c r="B210" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="211" spans="2:2">
       <c r="B211" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
     </row>
     <row r="212" spans="2:2">
       <c r="B212" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
     </row>
     <row r="213" spans="2:2">
       <c r="B213" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="214" spans="2:2">
       <c r="B214" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="215" spans="2:2">
       <c r="B215" t="s">
-        <v>657</v>
+        <v>374</v>
       </c>
     </row>
     <row r="216" spans="2:2">
       <c r="B216" t="s">
-        <v>660</v>
+        <v>657</v>
       </c>
     </row>
     <row r="217" spans="2:2">
       <c r="B217" t="s">
-        <v>377</v>
+        <v>660</v>
       </c>
     </row>
     <row r="218" spans="2:2">
       <c r="B218" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
     </row>
     <row r="219" spans="2:2">
       <c r="B219" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="220" spans="2:2">
       <c r="B220" t="s">
-        <v>740</v>
+        <v>380</v>
       </c>
     </row>
     <row r="221" spans="2:2">
       <c r="B221" t="s">
-        <v>382</v>
+        <v>744</v>
       </c>
     </row>
     <row r="222" spans="2:2">
       <c r="B222" t="s">
-        <v>753</v>
+        <v>382</v>
       </c>
     </row>
     <row r="223" spans="2:2">
       <c r="B223" t="s">
-        <v>384</v>
+        <v>757</v>
       </c>
     </row>
     <row r="224" spans="2:2">
       <c r="B224" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="225" spans="2:2">
       <c r="B225" t="s">
-        <v>388</v>
+        <v>386</v>
       </c>
     </row>
     <row r="226" spans="2:2">
       <c r="B226" t="s">
-        <v>390</v>
+        <v>388</v>
       </c>
     </row>
     <row r="227" spans="2:2">
       <c r="B227" t="s">
-        <v>392</v>
+        <v>390</v>
       </c>
     </row>
     <row r="228" spans="2:2">
       <c r="B228" t="s">
-        <v>394</v>
+        <v>392</v>
       </c>
     </row>
     <row r="229" spans="2:2">
       <c r="B229" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="230" spans="2:2">
       <c r="B230" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
     </row>
     <row r="231" spans="2:2">
       <c r="B231" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="232" spans="2:2">
       <c r="B232" t="s">
-        <v>663</v>
+        <v>400</v>
       </c>
     </row>
     <row r="233" spans="2:2">
       <c r="B233" t="s">
-        <v>666</v>
+        <v>663</v>
       </c>
     </row>
     <row r="234" spans="2:2">
       <c r="B234" t="s">
-        <v>402</v>
+        <v>666</v>
       </c>
     </row>
     <row r="235" spans="2:2">
       <c r="B235" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
     </row>
     <row r="236" spans="2:2">
       <c r="B236" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="237" spans="2:2">
       <c r="B237" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
     </row>
     <row r="238" spans="2:2">
       <c r="B238" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
     </row>
     <row r="239" spans="2:2">
       <c r="B239" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
     </row>
     <row r="240" spans="2:2">
       <c r="B240" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
     </row>
     <row r="241" spans="2:2">
       <c r="B241" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
     </row>
     <row r="242" spans="2:2">
       <c r="B242" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
     </row>
     <row r="243" spans="2:2">
       <c r="B243" t="s">
-        <v>710</v>
+        <v>420</v>
       </c>
     </row>
     <row r="244" spans="2:2">
       <c r="B244" t="s">
-        <v>669</v>
+        <v>710</v>
       </c>
     </row>
     <row r="245" spans="2:2">
       <c r="B245" t="s">
-        <v>421</v>
+        <v>669</v>
       </c>
     </row>
     <row r="246" spans="2:2">
       <c r="B246" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
     </row>
     <row r="247" spans="2:2">
       <c r="B247" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
     </row>
     <row r="248" spans="2:2">
       <c r="B248" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="249" spans="2:2">
       <c r="B249" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="250" spans="2:2">
       <c r="B250" t="s">
-        <v>671</v>
+        <v>429</v>
       </c>
     </row>
     <row r="251" spans="2:2">
       <c r="B251" t="s">
-        <v>431</v>
+        <v>671</v>
       </c>
     </row>
     <row r="252" spans="2:2">
       <c r="B252" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="253" spans="2:2">
       <c r="B253" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="254" spans="2:2">
       <c r="B254" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
     </row>
     <row r="255" spans="2:2">
       <c r="B255" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
     </row>
     <row r="256" spans="2:2">
       <c r="B256" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
     </row>
     <row r="257" spans="2:2">
       <c r="B257" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="258" spans="2:2">
       <c r="B258" t="s">
-        <v>446</v>
+        <v>444</v>
       </c>
     </row>
     <row r="259" spans="2:2">
       <c r="B259" t="s">
-        <v>448</v>
+        <v>446</v>
       </c>
     </row>
     <row r="260" spans="2:2">
       <c r="B260" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="261" spans="2:2">
       <c r="B261" t="s">
-        <v>673</v>
+        <v>450</v>
       </c>
     </row>
     <row r="262" spans="2:2">
       <c r="B262" t="s">
-        <v>452</v>
+        <v>673</v>
       </c>
     </row>
     <row r="263" spans="2:2">
       <c r="B263" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="264" spans="2:2">
       <c r="B264" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="265" spans="2:2">
       <c r="B265" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="266" spans="2:2">
       <c r="B266" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="267" spans="2:2">
       <c r="B267" t="s">
-        <v>676</v>
+        <v>460</v>
       </c>
     </row>
     <row r="268" spans="2:2">
       <c r="B268" t="s">
-        <v>462</v>
+        <v>676</v>
       </c>
     </row>
     <row r="269" spans="2:2">
       <c r="B269" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
     </row>
     <row r="270" spans="2:2">
       <c r="B270" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="271" spans="2:2">
       <c r="B271" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="272" spans="2:2">
       <c r="B272" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="273" spans="2:2">
       <c r="B273" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
     </row>
     <row r="274" spans="2:2">
       <c r="B274" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="275" spans="2:2">
       <c r="B275" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
     </row>
     <row r="276" spans="2:2">
       <c r="B276" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="277" spans="2:2">
       <c r="B277" t="s">
-        <v>479</v>
+        <v>477</v>
       </c>
     </row>
     <row r="278" spans="2:2">
       <c r="B278" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
     </row>
     <row r="279" spans="2:2">
       <c r="B279" t="s">
-        <v>483</v>
+        <v>481</v>
       </c>
     </row>
     <row r="280" spans="2:2">
       <c r="B280" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="281" spans="2:2">
       <c r="B281" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="282" spans="2:2">
       <c r="B282" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="283" spans="2:2">
       <c r="B283" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="284" spans="2:2">
       <c r="B284" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
     </row>
     <row r="285" spans="2:2">
       <c r="B285" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
     </row>
     <row r="286" spans="2:2">
       <c r="B286" t="s">
-        <v>498</v>
+        <v>495</v>
       </c>
     </row>
     <row r="287" spans="2:2">
       <c r="B287" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
     </row>
     <row r="288" spans="2:2">
       <c r="B288" t="s">
-        <v>503</v>
+        <v>500</v>
       </c>
     </row>
     <row r="289" spans="2:2">
       <c r="B289" t="s">
-        <v>757</v>
+        <v>503</v>
       </c>
     </row>
     <row r="290" spans="2:2">
@@ -9215,326 +9282,341 @@
     </row>
     <row r="291" spans="2:2">
       <c r="B291" t="s">
-        <v>505</v>
+        <v>765</v>
       </c>
     </row>
     <row r="292" spans="2:2">
       <c r="B292" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
     </row>
     <row r="293" spans="2:2">
       <c r="B293" t="s">
-        <v>763</v>
+        <v>507</v>
       </c>
     </row>
     <row r="294" spans="2:2">
       <c r="B294" t="s">
-        <v>679</v>
+        <v>767</v>
       </c>
     </row>
     <row r="295" spans="2:2">
       <c r="B295" t="s">
-        <v>509</v>
+        <v>679</v>
       </c>
     </row>
     <row r="296" spans="2:2">
       <c r="B296" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
     </row>
     <row r="297" spans="2:2">
       <c r="B297" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="298" spans="2:2">
       <c r="B298" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="299" spans="2:2">
       <c r="B299" t="s">
-        <v>712</v>
+        <v>515</v>
       </c>
     </row>
     <row r="300" spans="2:2">
       <c r="B300" t="s">
-        <v>517</v>
+        <v>712</v>
       </c>
     </row>
     <row r="301" spans="2:2">
       <c r="B301" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="302" spans="2:2">
       <c r="B302" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="303" spans="2:2">
       <c r="B303" t="s">
-        <v>714</v>
+        <v>521</v>
       </c>
     </row>
     <row r="304" spans="2:2">
       <c r="B304" t="s">
-        <v>523</v>
+        <v>714</v>
       </c>
     </row>
     <row r="305" spans="2:2">
       <c r="B305" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="306" spans="2:2">
       <c r="B306" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="307" spans="2:2">
       <c r="B307" t="s">
-        <v>529</v>
+        <v>527</v>
       </c>
     </row>
     <row r="308" spans="2:2">
       <c r="B308" t="s">
-        <v>531</v>
+        <v>529</v>
       </c>
     </row>
     <row r="309" spans="2:2">
       <c r="B309" t="s">
-        <v>533</v>
+        <v>531</v>
       </c>
     </row>
     <row r="310" spans="2:2">
       <c r="B310" t="s">
-        <v>716</v>
+        <v>533</v>
       </c>
     </row>
     <row r="311" spans="2:2">
       <c r="B311" t="s">
-        <v>535</v>
+        <v>716</v>
       </c>
     </row>
     <row r="312" spans="2:2">
       <c r="B312" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
     </row>
     <row r="313" spans="2:2">
       <c r="B313" t="s">
-        <v>539</v>
+        <v>537</v>
       </c>
     </row>
     <row r="314" spans="2:2">
       <c r="B314" t="s">
-        <v>541</v>
+        <v>539</v>
       </c>
     </row>
     <row r="315" spans="2:2">
       <c r="B315" t="s">
-        <v>543</v>
+        <v>541</v>
       </c>
     </row>
     <row r="316" spans="2:2">
       <c r="B316" t="s">
-        <v>545</v>
+        <v>543</v>
       </c>
     </row>
     <row r="317" spans="2:2">
       <c r="B317" t="s">
-        <v>547</v>
+        <v>545</v>
       </c>
     </row>
     <row r="318" spans="2:2">
       <c r="B318" t="s">
-        <v>549</v>
+        <v>547</v>
       </c>
     </row>
     <row r="319" spans="2:2">
       <c r="B319" t="s">
-        <v>551</v>
+        <v>549</v>
       </c>
     </row>
     <row r="320" spans="2:2">
       <c r="B320" t="s">
-        <v>553</v>
+        <v>551</v>
       </c>
     </row>
     <row r="321" spans="2:2">
       <c r="B321" t="s">
-        <v>555</v>
+        <v>553</v>
       </c>
     </row>
     <row r="322" spans="2:2">
       <c r="B322" t="s">
-        <v>557</v>
+        <v>555</v>
       </c>
     </row>
     <row r="323" spans="2:2">
       <c r="B323" t="s">
-        <v>682</v>
+        <v>557</v>
       </c>
     </row>
     <row r="324" spans="2:2">
       <c r="B324" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="325" spans="2:2">
       <c r="B325" t="s">
-        <v>687</v>
+        <v>684</v>
       </c>
     </row>
     <row r="326" spans="2:2">
       <c r="B326" t="s">
-        <v>559</v>
+        <v>687</v>
       </c>
     </row>
     <row r="327" spans="2:2">
       <c r="B327" t="s">
-        <v>561</v>
+        <v>559</v>
       </c>
     </row>
     <row r="328" spans="2:2">
       <c r="B328" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="329" spans="2:2">
       <c r="B329" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
     </row>
     <row r="330" spans="2:2">
       <c r="B330" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
     </row>
     <row r="331" spans="2:2">
       <c r="B331" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
     </row>
     <row r="332" spans="2:2">
       <c r="B332" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
     </row>
     <row r="333" spans="2:2">
       <c r="B333" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="334" spans="2:2">
       <c r="B334" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
     </row>
     <row r="335" spans="2:2">
       <c r="B335" t="s">
-        <v>743</v>
+        <v>575</v>
       </c>
     </row>
     <row r="336" spans="2:2">
       <c r="B336" t="s">
-        <v>577</v>
+        <v>747</v>
       </c>
     </row>
     <row r="337" spans="1:2">
       <c r="B337" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
     </row>
     <row r="338" spans="1:2">
       <c r="B338" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
     </row>
     <row r="339" spans="1:2">
       <c r="B339" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="340" spans="1:2">
       <c r="B340" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
     </row>
     <row r="341" spans="1:2">
       <c r="B341" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
     </row>
     <row r="342" spans="1:2">
       <c r="B342" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="343" spans="1:2">
       <c r="B343" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="344" spans="1:2">
       <c r="B344" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
     </row>
     <row r="345" spans="1:2">
       <c r="B345" t="s">
-        <v>596</v>
+        <v>593</v>
       </c>
     </row>
     <row r="346" spans="1:2">
       <c r="B346" t="s">
+        <v>596</v>
+      </c>
+    </row>
+    <row r="347" spans="1:2">
+      <c r="B347" t="s">
         <v>598</v>
       </c>
     </row>
-    <row r="348" spans="1:2">
-      <c r="A348" t="s">
-        <v>769</v>
-      </c>
-      <c r="B348" t="s">
-        <v>696</v>
+    <row r="349" spans="1:2">
+      <c r="A349" t="s">
+        <v>773</v>
+      </c>
+      <c r="B349" t="s">
+        <v>731</v>
       </c>
     </row>
     <row r="350" spans="1:2">
-      <c r="A350" t="s">
-        <v>770</v>
-      </c>
       <c r="B350" t="s">
-        <v>616</v>
+        <v>731</v>
       </c>
     </row>
     <row r="351" spans="1:2">
       <c r="B351" t="s">
-        <v>676</v>
+        <v>619</v>
+      </c>
+    </row>
+    <row r="352" spans="1:2">
+      <c r="B352" t="s">
+        <v>740</v>
       </c>
     </row>
     <row r="353" spans="1:2">
-      <c r="A353" t="s">
-        <v>771</v>
-      </c>
       <c r="B353" t="s">
-        <v>619</v>
+        <v>633</v>
       </c>
     </row>
     <row r="354" spans="1:2">
       <c r="B354" t="s">
-        <v>736</v>
-      </c>
-    </row>
-    <row r="355" spans="1:2">
-      <c r="B355" t="s">
-        <v>633</v>
+        <v>644</v>
       </c>
     </row>
     <row r="356" spans="1:2">
+      <c r="A356" t="s">
+        <v>774</v>
+      </c>
       <c r="B356" t="s">
-        <v>644</v>
+        <v>696</v>
+      </c>
+    </row>
+    <row r="358" spans="1:2">
+      <c r="A358" t="s">
+        <v>775</v>
+      </c>
+      <c r="B358" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="359" spans="1:2">
+      <c r="B359" t="s">
+        <v>676</v>
       </c>
     </row>
   </sheetData>
@@ -10511,6 +10593,60 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="3" max="3" width="110.7109375" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>731</v>
+      </c>
+      <c r="B3">
+        <v>1.45</v>
+      </c>
+      <c r="C3" t="s">
+        <v>732</v>
+      </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>733</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -10521,7 +10657,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10543,47 +10679,47 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="B3">
         <v>1.9</v>
       </c>
       <c r="C3" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="B4">
         <v>2.11</v>
       </c>
       <c r="C4" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="D4" t="s">
         <v>8</v>
       </c>
       <c r="E4" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="B5">
         <v>2.7</v>
       </c>
       <c r="C5" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>
@@ -10594,13 +10730,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="B6">
         <v>2.58</v>
       </c>
       <c r="C6" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="D6" t="s">
         <v>8</v>
@@ -10611,90 +10747,36 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B7">
         <v>1.93</v>
       </c>
       <c r="C7" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="D7" t="s">
         <v>8</v>
       </c>
       <c r="E7" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="B8">
         <v>2.05</v>
       </c>
       <c r="C8" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="D8" t="s">
         <v>8</v>
       </c>
       <c r="E8" t="s">
         <v>612</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="3" max="3" width="110.7109375" customWidth="1"/>
-    <col min="4" max="4" width="20.7109375" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5">
-      <c r="A1" t="s">
-        <v>745</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D2" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>746</v>
-      </c>
-      <c r="B3">
-        <v>0.93</v>
-      </c>
-      <c r="C3" t="s">
-        <v>747</v>
-      </c>
-      <c r="D3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E3" t="s">
-        <v>443</v>
       </c>
     </row>
   </sheetData>
@@ -10714,7 +10796,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -10736,19 +10818,19 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="B3">
-        <v>2.17</v>
+        <v>0.93</v>
       </c>
       <c r="C3" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
       <c r="E3" t="s">
-        <v>751</v>
+        <v>443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>